<commit_message>
BSD-Catalog-Master - preturi aplicate automat (1199-1999 lei)
</commit_message>
<xml_diff>
--- a/BSD-Catalog-Master.xlsx
+++ b/BSD-Catalog-Master.xlsx
@@ -31,7 +31,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -108,6 +108,16 @@
         <fgColor rgb="002E7D32"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -121,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -153,6 +163,12 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -612,8 +628,12 @@
           <t>Unghi mort Mercedes-Benz C-Class W204 2007-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+      <c r="C3" s="29" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D3" s="30" t="n">
+        <v>950</v>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -652,8 +672,12 @@
           <t>Unghi mort Mercedes-Benz E-Class W212 2009-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr"/>
+      <c r="C4" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D4" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -692,8 +716,12 @@
           <t>Unghi mort Mercedes-Benz GLK X204 2008-2015 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
+      <c r="C5" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D5" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -732,8 +760,12 @@
           <t>Unghi mort Mercedes-Benz GLA X156 2013-2020 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr"/>
+      <c r="C6" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D6" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -772,8 +804,12 @@
           <t>Unghi mort Mercedes-Benz A-Class W176 2012-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
+      <c r="C7" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D7" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -812,8 +848,12 @@
           <t>Unghi mort Mercedes-Benz B-Class W246 2011-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr"/>
+      <c r="C8" s="29" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D8" s="30" t="n">
+        <v>950</v>
+      </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -852,8 +892,12 @@
           <t>Unghi mort Mercedes-Benz CLA C117 2013-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+      <c r="C9" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D9" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -892,8 +936,12 @@
           <t>Unghi mort Mercedes-Benz S-Class W221 2005-2013 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr"/>
+      <c r="C10" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D10" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -932,8 +980,12 @@
           <t>Unghi mort Mercedes-Benz CLS C218 2011-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+      <c r="C11" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D11" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -972,8 +1024,12 @@
           <t>Unghi mort Mercedes-Benz ML W164 2005-2011 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="4" t="inlineStr"/>
+      <c r="C12" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D12" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1012,8 +1068,12 @@
           <t>Unghi mort Mercedes-Benz GLE W166 2015-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+      <c r="C13" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D13" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1052,8 +1112,12 @@
           <t>Unghi mort Mercedes-Benz GLS X166 2015-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr"/>
+      <c r="C14" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D14" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1092,8 +1156,12 @@
           <t>Unghi mort Mercedes-Benz GL X166 2012-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+      <c r="C15" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D15" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1132,8 +1200,12 @@
           <t>Unghi mort Mercedes-Benz R-Class W251 2005-2017 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="4" t="inlineStr"/>
+      <c r="C16" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D16" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1172,8 +1244,12 @@
           <t>Unghi mort Mercedes-Benz G-Class W463 2008-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
+      <c r="C17" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D17" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1212,8 +1288,12 @@
           <t>Unghi mort Mercedes-Benz C-Class W205 2014-2021 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
+      <c r="C18" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D18" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1252,8 +1332,12 @@
           <t>Unghi mort Mercedes-Benz E-Class W213 2016-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
+      <c r="C19" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D19" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E19" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1292,8 +1376,12 @@
           <t>Unghi mort Mercedes-Benz GLA H247 2020-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr"/>
-      <c r="D20" s="4" t="inlineStr"/>
+      <c r="C20" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D20" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1332,8 +1420,12 @@
           <t>Unghi mort Mercedes-Benz GLC X253 2015-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+      <c r="C21" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D21" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1372,8 +1464,12 @@
           <t>Unghi mort Mercedes-Benz GLB X247 2019-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="4" t="inlineStr"/>
+      <c r="C22" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D22" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1412,8 +1508,12 @@
           <t>Unghi mort Mercedes-Benz B-Class W247 2018-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
+      <c r="C23" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D23" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1452,8 +1552,12 @@
           <t>Unghi mort Mercedes-Benz EQC N293 2019-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="4" t="inlineStr"/>
+      <c r="C24" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D24" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1492,8 +1596,12 @@
           <t>Unghi mort Mercedes-Benz EQA H243 2021-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
+      <c r="C25" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D25" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1532,8 +1640,12 @@
           <t>Unghi mort Mercedes-Benz EQB X243 2021-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr"/>
+      <c r="C26" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D26" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1572,8 +1684,12 @@
           <t>Unghi mort Mercedes-Benz S-Class W222 2013-2020 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
+      <c r="C27" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D27" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1612,8 +1728,12 @@
           <t>Unghi mort Mercedes-Benz CLS C257 2018-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="4" t="inlineStr"/>
+      <c r="C28" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D28" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1652,8 +1772,12 @@
           <t>Unghi mort Mercedes-Benz GT AMG C190 2014-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
+      <c r="C29" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D29" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1692,8 +1816,12 @@
           <t>Unghi mort Mercedes-Benz A-Class W177 2018-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="4" t="inlineStr"/>
+      <c r="C30" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D30" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1732,8 +1860,12 @@
           <t>Unghi mort Mercedes-Benz CLA C118 2019-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
+      <c r="C31" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D31" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1772,8 +1904,12 @@
           <t>Unghi mort Mercedes-Benz Vito W447 2014-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr"/>
-      <c r="D32" s="4" t="inlineStr"/>
+      <c r="C32" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D32" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1812,8 +1948,12 @@
           <t>Unghi mort Mercedes-Benz V-Class W447 2014-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
+      <c r="C33" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D33" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1852,8 +1992,12 @@
           <t>Unghi mort Mercedes-Benz EQV W447 2020-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr"/>
+      <c r="C34" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D34" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1892,8 +2036,12 @@
           <t>Unghi mort Mercedes-Benz G-Class W463 2012-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
+      <c r="C35" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D35" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1932,8 +2080,12 @@
           <t>Unghi mort Mercedes-Benz C-Class W206 2021-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr"/>
-      <c r="D36" s="4" t="inlineStr"/>
+      <c r="C36" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D36" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -1972,8 +2124,12 @@
           <t>Unghi mort Mercedes-Benz GLC X254 2022-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
+      <c r="C37" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D37" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2012,8 +2168,12 @@
           <t>Unghi mort Mercedes-Benz EQS V297 2021-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr"/>
-      <c r="D38" s="4" t="inlineStr"/>
+      <c r="C38" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D38" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2052,8 +2212,12 @@
           <t>Unghi mort Mercedes-Benz E-Class W214 2023-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
+      <c r="C39" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D39" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2092,8 +2256,12 @@
           <t>Unghi mort Mercedes-Benz S-Class W223 2020-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="4" t="inlineStr"/>
+      <c r="C40" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D40" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2132,8 +2300,12 @@
           <t>Unghi mort Mercedes-Benz S Maybach W223 2020-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
+      <c r="C41" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D41" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2172,8 +2344,12 @@
           <t>Unghi mort Mercedes-Benz CLE W236 2023-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr"/>
-      <c r="D42" s="4" t="inlineStr"/>
+      <c r="C42" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D42" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2212,8 +2388,12 @@
           <t>Unghi mort Mercedes-Benz GLE V167 2018-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
+      <c r="C43" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D43" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2252,8 +2432,12 @@
           <t>Unghi mort Mercedes-Benz GLS X167 2019-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr"/>
-      <c r="D44" s="4" t="inlineStr"/>
+      <c r="C44" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D44" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2292,8 +2476,12 @@
           <t>Unghi mort Mercedes-Benz G-Class W463 2018-2026 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
+      <c r="C45" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D45" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2348,8 +2536,12 @@
           <t>Unghi mort Audi A6L 2012-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
+      <c r="C47" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D47" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2388,8 +2580,12 @@
           <t>Unghi mort Audi S6 2013-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr"/>
-      <c r="D48" s="4" t="inlineStr"/>
+      <c r="C48" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D48" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2428,8 +2624,12 @@
           <t>Unghi mort Audi A6 2013-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
+      <c r="C49" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D49" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2468,8 +2668,12 @@
           <t>Unghi mort Audi A4L 2017-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr"/>
-      <c r="D50" s="4" t="inlineStr"/>
+      <c r="C50" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D50" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2508,8 +2712,12 @@
           <t>Unghi mort Audi A5 2017-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
+      <c r="C51" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D51" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2548,8 +2756,12 @@
           <t>Unghi mort Audi RS4 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr"/>
-      <c r="D52" s="4" t="inlineStr"/>
+      <c r="C52" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D52" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2588,8 +2800,12 @@
           <t>Unghi mort Audi RS5 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
+      <c r="C53" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D53" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E53" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2628,8 +2844,12 @@
           <t>Unghi mort Audi A4 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr"/>
-      <c r="D54" s="4" t="inlineStr"/>
+      <c r="C54" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D54" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2668,8 +2888,12 @@
           <t>Unghi mort Audi S4 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
+      <c r="C55" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D55" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2708,8 +2932,12 @@
           <t>Unghi mort Audi S5 2017-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr"/>
-      <c r="D56" s="4" t="inlineStr"/>
+      <c r="C56" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D56" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2748,8 +2976,12 @@
           <t>Unghi mort Audi A3 2014-2020 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
+      <c r="C57" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D57" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E57" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2788,8 +3020,12 @@
           <t>Unghi mort Audi S3 2015-2020 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr"/>
-      <c r="D58" s="4" t="inlineStr"/>
+      <c r="C58" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D58" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2828,8 +3064,12 @@
           <t>Unghi mort Audi A6L 2009-2011 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
+      <c r="C59" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D59" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E59" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2868,8 +3108,12 @@
           <t>Unghi mort Audi Q3 2012-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr"/>
-      <c r="D60" s="4" t="inlineStr"/>
+      <c r="C60" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D60" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2908,8 +3152,12 @@
           <t>Unghi mort Audi A8 2008-2009 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
+      <c r="C61" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D61" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2948,8 +3196,12 @@
           <t>Unghi mort Audi A4L 2009-2012 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr"/>
-      <c r="D62" s="4" t="inlineStr"/>
+      <c r="C62" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D62" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -2988,8 +3240,12 @@
           <t>Unghi mort Audi A4 2013-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
+      <c r="C63" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D63" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E63" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3028,8 +3284,12 @@
           <t>Unghi mort Audi A4L 2013-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C64" s="4" t="inlineStr"/>
-      <c r="D64" s="4" t="inlineStr"/>
+      <c r="C64" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D64" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3068,8 +3328,12 @@
           <t>Unghi mort Audi A5 2012-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
+      <c r="C65" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D65" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E65" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3108,8 +3372,12 @@
           <t>Unghi mort Audi S5 2010-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr"/>
-      <c r="D66" s="4" t="inlineStr"/>
+      <c r="C66" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D66" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3148,8 +3416,12 @@
           <t>Unghi mort Audi A3 2013-2013 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
+      <c r="C67" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D67" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E67" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3188,8 +3460,12 @@
           <t>Unghi mort Audi RS5 2011-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr"/>
-      <c r="D68" s="4" t="inlineStr"/>
+      <c r="C68" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D68" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3228,8 +3504,12 @@
           <t>Unghi mort Audi Q5 2010-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
+      <c r="C69" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D69" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E69" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3268,8 +3548,12 @@
           <t>Unghi mort Audi SQ5 2010-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr"/>
-      <c r="D70" s="4" t="inlineStr"/>
+      <c r="C70" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D70" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3308,8 +3592,12 @@
           <t>Unghi mort Audi Q7 2006-2015 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
+      <c r="C71" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D71" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E71" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3348,8 +3636,12 @@
           <t>Unghi mort Audi Q7 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C72" s="4" t="inlineStr"/>
-      <c r="D72" s="4" t="inlineStr"/>
+      <c r="C72" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D72" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3388,8 +3680,12 @@
           <t>Unghi mort Audi Q5L 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
+      <c r="C73" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D73" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E73" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3428,8 +3724,12 @@
           <t>Unghi mort Audi Q2L 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C74" s="4" t="inlineStr"/>
-      <c r="D74" s="4" t="inlineStr"/>
+      <c r="C74" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D74" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3468,8 +3768,12 @@
           <t>Unghi mort Audi Q3 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
+      <c r="C75" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D75" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E75" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3508,8 +3812,12 @@
           <t>Unghi mort Audi A6L 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C76" s="4" t="inlineStr"/>
-      <c r="D76" s="4" t="inlineStr"/>
+      <c r="C76" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D76" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3548,8 +3856,12 @@
           <t>Unghi mort Audi A7 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr"/>
+      <c r="C77" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D77" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3588,8 +3900,12 @@
           <t>Unghi mort Audi A8L 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C78" s="4" t="inlineStr"/>
-      <c r="D78" s="4" t="inlineStr"/>
+      <c r="C78" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D78" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3628,8 +3944,12 @@
           <t>Unghi mort Audi A6 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr"/>
-      <c r="D79" t="inlineStr"/>
+      <c r="C79" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D79" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3668,8 +3988,12 @@
           <t>Unghi mort Audi RS7 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C80" s="4" t="inlineStr"/>
-      <c r="D80" s="4" t="inlineStr"/>
+      <c r="C80" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D80" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3708,8 +4032,12 @@
           <t>Unghi mort Audi S8 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr"/>
+      <c r="C81" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D81" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3748,8 +4076,12 @@
           <t>Unghi mort Audi A1 2012-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C82" s="4" t="inlineStr"/>
-      <c r="D82" s="4" t="inlineStr"/>
+      <c r="C82" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D82" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3788,8 +4120,12 @@
           <t>Unghi mort Audi A1 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr"/>
+      <c r="C83" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D83" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3828,8 +4164,12 @@
           <t>Unghi mort Audi A3 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C84" s="4" t="inlineStr"/>
-      <c r="D84" s="4" t="inlineStr"/>
+      <c r="C84" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D84" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3868,8 +4208,12 @@
           <t>Unghi mort Audi e-tron 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr"/>
+      <c r="C85" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D85" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3908,8 +4252,12 @@
           <t>Unghi mort Audi A8 2011-2017 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C86" s="4" t="inlineStr"/>
-      <c r="D86" s="4" t="inlineStr"/>
+      <c r="C86" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D86" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3948,8 +4296,12 @@
           <t>Unghi mort Audi S8 2013-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
-      <c r="D87" t="inlineStr"/>
+      <c r="C87" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D87" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -3988,8 +4340,12 @@
           <t>Unghi mort Audi Q6 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C88" s="4" t="inlineStr"/>
-      <c r="D88" s="4" t="inlineStr"/>
+      <c r="C88" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D88" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4028,8 +4384,12 @@
           <t>Unghi mort Audi Q8 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr"/>
+      <c r="C89" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D89" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4068,8 +4428,12 @@
           <t>Unghi mort Audi Q4 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C90" s="4" t="inlineStr"/>
-      <c r="D90" s="4" t="inlineStr"/>
+      <c r="C90" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D90" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4108,8 +4472,12 @@
           <t>Unghi mort Audi Q5 e-tron 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
-      <c r="D91" t="inlineStr"/>
+      <c r="C91" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D91" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4164,8 +4532,12 @@
           <t>Unghi mort BMW BMW 5 2011-2017 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
-      <c r="D93" t="inlineStr"/>
+      <c r="C93" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D93" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4204,8 +4576,12 @@
           <t>Unghi mort BMW BMW 7 2009-2015 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C94" s="4" t="inlineStr"/>
-      <c r="D94" s="4" t="inlineStr"/>
+      <c r="C94" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D94" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4244,8 +4620,12 @@
           <t>Unghi mort BMW BMW 5 GT 2010-2017 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr"/>
+      <c r="C95" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D95" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E95" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4284,8 +4664,12 @@
           <t>Unghi mort BMW BMW 6 2012-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C96" s="4" t="inlineStr"/>
-      <c r="D96" s="4" t="inlineStr"/>
+      <c r="C96" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D96" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4324,8 +4708,12 @@
           <t>Unghi mort BMW BMW 3 2013-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr"/>
+      <c r="C97" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D97" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E97" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4364,8 +4752,12 @@
           <t>Unghi mort BMW BMW X1 2013-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C98" s="4" t="inlineStr"/>
-      <c r="D98" s="4" t="inlineStr"/>
+      <c r="C98" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D98" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4404,8 +4796,12 @@
           <t>Unghi mort BMW BMW 4 2013-2020 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr"/>
+      <c r="C99" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D99" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4444,8 +4840,12 @@
           <t>Unghi mort BMW BMW 3 GT 2013-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C100" s="4" t="inlineStr"/>
-      <c r="D100" s="4" t="inlineStr"/>
+      <c r="C100" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D100" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4484,8 +4884,12 @@
           <t>Unghi mort BMW BMW 2 2014-2021 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
-      <c r="D101" t="inlineStr"/>
+      <c r="C101" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D101" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4524,8 +4928,12 @@
           <t>Unghi mort BMW BMW 2 2018-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C102" s="4" t="inlineStr"/>
-      <c r="D102" s="4" t="inlineStr"/>
+      <c r="C102" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D102" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4564,8 +4972,12 @@
           <t>Unghi mort BMW BMW 1 2017-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr"/>
-      <c r="D103" t="inlineStr"/>
+      <c r="C103" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D103" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4604,8 +5016,12 @@
           <t>Unghi mort BMW BMW X2 2018-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C104" s="4" t="inlineStr"/>
-      <c r="D104" s="4" t="inlineStr"/>
+      <c r="C104" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D104" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4644,8 +5060,12 @@
           <t>Unghi mort BMW Z4 2019-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr"/>
-      <c r="D105" t="inlineStr"/>
+      <c r="C105" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D105" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4684,8 +5104,12 @@
           <t>Unghi mort BMW 2019 I3  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C106" s="4" t="inlineStr"/>
-      <c r="D106" s="4" t="inlineStr"/>
+      <c r="C106" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D106" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4720,8 +5144,12 @@
           <t>Unghi mort BMW X3 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
-      <c r="D107" t="inlineStr"/>
+      <c r="C107" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D107" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4760,8 +5188,12 @@
           <t>Unghi mort BMW X4 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C108" s="4" t="inlineStr"/>
-      <c r="D108" s="4" t="inlineStr"/>
+      <c r="C108" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D108" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4800,8 +5232,12 @@
           <t>Unghi mort BMW X5 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr"/>
-      <c r="D109" t="inlineStr"/>
+      <c r="C109" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D109" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E109" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4840,8 +5276,12 @@
           <t>Unghi mort BMW X6 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C110" s="4" t="inlineStr"/>
-      <c r="D110" s="4" t="inlineStr"/>
+      <c r="C110" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D110" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4880,8 +5320,12 @@
           <t>Unghi mort BMW X7 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr"/>
-      <c r="D111" t="inlineStr"/>
+      <c r="C111" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D111" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E111" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4920,8 +5364,12 @@
           <t>Unghi mort BMW IX3 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C112" s="4" t="inlineStr"/>
-      <c r="D112" s="4" t="inlineStr"/>
+      <c r="C112" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D112" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -4960,8 +5408,12 @@
           <t>Unghi mort BMW X4M 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr"/>
-      <c r="D113" t="inlineStr"/>
+      <c r="C113" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D113" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E113" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5000,8 +5452,12 @@
           <t>Unghi mort BMW X3M 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C114" s="4" t="inlineStr"/>
-      <c r="D114" s="4" t="inlineStr"/>
+      <c r="C114" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D114" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5040,8 +5496,12 @@
           <t>Unghi mort BMW X5M 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr"/>
-      <c r="D115" t="inlineStr"/>
+      <c r="C115" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D115" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E115" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5080,8 +5540,12 @@
           <t>Unghi mort BMW X6M 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C116" s="4" t="inlineStr"/>
-      <c r="D116" s="4" t="inlineStr"/>
+      <c r="C116" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D116" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5120,8 +5584,12 @@
           <t>Unghi mort BMW BMW 7 2016-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr"/>
-      <c r="D117" t="inlineStr"/>
+      <c r="C117" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D117" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E117" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5160,8 +5628,12 @@
           <t>Unghi mort BMW BMW 5 2018-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C118" s="4" t="inlineStr"/>
-      <c r="D118" s="4" t="inlineStr"/>
+      <c r="C118" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D118" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5200,8 +5672,12 @@
           <t>Unghi mort BMW BMW 4 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
-      <c r="D119" t="inlineStr"/>
+      <c r="C119" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D119" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E119" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5240,8 +5716,12 @@
           <t>Unghi mort BMW BMW 6 GT 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C120" s="4" t="inlineStr"/>
-      <c r="D120" s="4" t="inlineStr"/>
+      <c r="C120" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D120" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5280,8 +5760,12 @@
           <t>Unghi mort BMW BMW 3 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr"/>
-      <c r="D121" t="inlineStr"/>
+      <c r="C121" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D121" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E121" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5320,8 +5804,12 @@
           <t>Unghi mort BMW BMW 8 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C122" s="4" t="inlineStr"/>
-      <c r="D122" s="4" t="inlineStr"/>
+      <c r="C122" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D122" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5360,8 +5848,12 @@
           <t>Unghi mort BMW BMW 2 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr"/>
-      <c r="D123" t="inlineStr"/>
+      <c r="C123" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D123" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E123" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5400,8 +5892,12 @@
           <t>Unghi mort BMW BMW M4 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C124" s="4" t="inlineStr"/>
-      <c r="D124" s="4" t="inlineStr"/>
+      <c r="C124" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D124" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5440,8 +5936,12 @@
           <t>Unghi mort BMW BMW I3 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr"/>
-      <c r="D125" t="inlineStr"/>
+      <c r="C125" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D125" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E125" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5480,8 +5980,12 @@
           <t>Unghi mort BMW BMW I4 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C126" s="4" t="inlineStr"/>
-      <c r="D126" s="4" t="inlineStr"/>
+      <c r="C126" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D126" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5520,8 +6024,12 @@
           <t>Unghi mort BMW BMW M3 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr"/>
-      <c r="D127" t="inlineStr"/>
+      <c r="C127" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D127" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E127" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5560,8 +6068,12 @@
           <t>Unghi mort BMW 2019  BMW M8  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C128" s="4" t="inlineStr"/>
-      <c r="D128" s="4" t="inlineStr"/>
+      <c r="C128" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D128" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5596,8 +6108,12 @@
           <t>Unghi mort BMW BMW M5 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr"/>
-      <c r="D129" t="inlineStr"/>
+      <c r="C129" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D129" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E129" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5636,8 +6152,12 @@
           <t>Unghi mort BMW MINI 2015-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C130" s="4" t="inlineStr"/>
-      <c r="D130" s="4" t="inlineStr"/>
+      <c r="C130" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D130" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5676,8 +6196,12 @@
           <t>Unghi mort BMW MINI CLUBMAN 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr"/>
-      <c r="D131" t="inlineStr"/>
+      <c r="C131" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D131" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E131" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5716,8 +6240,12 @@
           <t>Unghi mort BMW MINI COUNTRYMAN 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C132" s="4" t="inlineStr"/>
-      <c r="D132" s="4" t="inlineStr"/>
+      <c r="C132" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D132" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5756,8 +6284,12 @@
           <t>Unghi mort BMW 2023 BMW 7  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr"/>
-      <c r="D133" t="inlineStr"/>
+      <c r="C133" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D133" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E133" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5790,8 +6322,12 @@
           <t>Unghi mort BMW 2024 BMW 5  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C134" s="4" t="inlineStr"/>
-      <c r="D134" s="4" t="inlineStr"/>
+      <c r="C134" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D134" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5826,8 +6362,12 @@
           <t>Unghi mort BMW 2023 BMW I7  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr"/>
-      <c r="D135" t="inlineStr"/>
+      <c r="C135" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D135" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E135" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5860,8 +6400,12 @@
           <t>Unghi mort BMW X5 2008-2013 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C136" s="4" t="inlineStr"/>
-      <c r="D136" s="4" t="inlineStr"/>
+      <c r="C136" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D136" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5900,8 +6444,12 @@
           <t>Unghi mort BMW X6 2009-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr"/>
-      <c r="D137" t="inlineStr"/>
+      <c r="C137" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D137" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E137" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5940,8 +6488,12 @@
           <t>Unghi mort BMW 2O1O-2014 X5M  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C138" s="4" t="inlineStr"/>
-      <c r="D138" s="4" t="inlineStr"/>
+      <c r="C138" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D138" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -5976,8 +6528,12 @@
           <t>Unghi mort BMW X6M 2013-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr"/>
-      <c r="D139" t="inlineStr"/>
+      <c r="C139" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D139" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E139" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6016,8 +6572,12 @@
           <t>Unghi mort BMW 2013 C5  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C140" s="4" t="inlineStr"/>
-      <c r="D140" s="4" t="inlineStr"/>
+      <c r="C140" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D140" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6068,8 +6628,12 @@
           <t>Unghi mort Toyota Wildlander 2020-2025 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C142" s="4" t="inlineStr"/>
-      <c r="D142" s="4" t="inlineStr"/>
+      <c r="C142" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D142" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6108,8 +6672,12 @@
           <t>Unghi mort Toyota Frontlander 2022-2025 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr"/>
-      <c r="D143" t="inlineStr"/>
+      <c r="C143" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D143" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E143" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6148,8 +6716,12 @@
           <t>Unghi mort Toyota Venza 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C144" s="4" t="inlineStr"/>
-      <c r="D144" s="4" t="inlineStr"/>
+      <c r="C144" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D144" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6188,8 +6760,12 @@
           <t>Unghi mort Toyota Rav4 2020-2025 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr"/>
-      <c r="D145" t="inlineStr"/>
+      <c r="C145" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D145" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E145" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6228,8 +6804,12 @@
           <t>Unghi mort Toyota Toyota cross 2022-2025 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C146" s="4" t="inlineStr"/>
-      <c r="D146" s="4" t="inlineStr"/>
+      <c r="C146" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D146" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6268,8 +6848,12 @@
           <t>Unghi mort Toyota Toyota Hilux 2021-2025 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr"/>
-      <c r="D147" t="inlineStr"/>
+      <c r="C147" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D147" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E147" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6308,8 +6892,12 @@
           <t>Unghi mort Toyota CROWN KLUGER 2021-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C148" s="4" t="inlineStr"/>
-      <c r="D148" s="4" t="inlineStr"/>
+      <c r="C148" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D148" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6348,8 +6936,12 @@
           <t>Unghi mort Toyota Highlander 2015-2021 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr"/>
-      <c r="D149" t="inlineStr"/>
+      <c r="C149" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D149" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E149" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6388,8 +6980,12 @@
           <t>Unghi mort Toyota Toyota Alphard 30 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C150" s="4" t="inlineStr"/>
-      <c r="D150" s="4" t="inlineStr"/>
+      <c r="C150" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D150" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6428,8 +7024,12 @@
           <t>Unghi mort Toyota Toyota Vellfire 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr"/>
-      <c r="D151" t="inlineStr"/>
+      <c r="C151" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D151" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E151" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6468,8 +7068,12 @@
           <t>Unghi mort Toyota 4 Runner 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C152" s="4" t="inlineStr"/>
-      <c r="D152" s="4" t="inlineStr"/>
+      <c r="C152" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D152" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6508,8 +7112,12 @@
           <t>Unghi mort Toyota Fortuner 2015-2025 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr"/>
-      <c r="D153" t="inlineStr"/>
+      <c r="C153" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D153" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E153" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6548,8 +7156,12 @@
           <t>Unghi mort Toyota Tacoma 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C154" s="4" t="inlineStr"/>
-      <c r="D154" s="4" t="inlineStr"/>
+      <c r="C154" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D154" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6588,8 +7200,12 @@
           <t>Unghi mort Toyota Highlander 2022-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr"/>
-      <c r="D155" t="inlineStr"/>
+      <c r="C155" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D155" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E155" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6628,8 +7244,12 @@
           <t>Unghi mort Toyota Sienna 2021-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C156" s="4" t="inlineStr"/>
-      <c r="D156" s="4" t="inlineStr"/>
+      <c r="C156" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D156" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6668,8 +7288,12 @@
           <t>Unghi mort Toyota Verso 2009-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr"/>
-      <c r="D157" t="inlineStr"/>
+      <c r="C157" s="29" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D157" s="30" t="n">
+        <v>950</v>
+      </c>
       <c r="E157" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6708,8 +7332,12 @@
           <t>Unghi mort Toyota Rav4 2009-2012 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C158" s="4" t="inlineStr"/>
-      <c r="D158" s="4" t="inlineStr"/>
+      <c r="C158" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D158" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6748,8 +7376,12 @@
           <t>Unghi mort Toyota Corolla 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr"/>
-      <c r="D159" t="inlineStr"/>
+      <c r="C159" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D159" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E159" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6788,8 +7420,12 @@
           <t>Unghi mort Toyota Prado 2010-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C160" s="4" t="inlineStr"/>
-      <c r="D160" s="4" t="inlineStr"/>
+      <c r="C160" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D160" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6828,8 +7464,12 @@
           <t>Unghi mort Toyota Land Cruiser LC200 2010-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr"/>
-      <c r="D161" t="inlineStr"/>
+      <c r="C161" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D161" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E161" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6868,8 +7508,12 @@
           <t>Unghi mort Toyota Land Cruiser LC300 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C162" s="4" t="inlineStr"/>
-      <c r="D162" s="4" t="inlineStr"/>
+      <c r="C162" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D162" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6908,8 +7552,12 @@
           <t>Unghi mort Toyota Land Cruiser LC100 2007-2009 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr"/>
-      <c r="D163" t="inlineStr"/>
+      <c r="C163" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D163" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E163" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6948,8 +7596,12 @@
           <t>Unghi mort Toyota Rav4 2013-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C164" s="4" t="inlineStr"/>
-      <c r="D164" s="4" t="inlineStr"/>
+      <c r="C164" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D164" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -6988,8 +7640,12 @@
           <t>Unghi mort Toyota Corolla 2014-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr"/>
-      <c r="D165" t="inlineStr"/>
+      <c r="C165" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D165" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E165" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7028,8 +7684,12 @@
           <t>Unghi mort Toyota Camry 2009-2011 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C166" s="4" t="inlineStr"/>
-      <c r="D166" s="4" t="inlineStr"/>
+      <c r="C166" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D166" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7068,8 +7728,12 @@
           <t>Unghi mort Toyota Yaris 2009-2011 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr"/>
-      <c r="D167" t="inlineStr"/>
+      <c r="C167" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D167" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E167" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7108,8 +7772,12 @@
           <t>Unghi mort Toyota Corolla 2008-2013 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C168" s="4" t="inlineStr"/>
-      <c r="D168" s="4" t="inlineStr"/>
+      <c r="C168" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D168" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7148,8 +7816,12 @@
           <t>Unghi mort Toyota 2010 Prius  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr"/>
-      <c r="D169" t="inlineStr"/>
+      <c r="C169" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D169" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E169" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7182,8 +7854,12 @@
           <t>Unghi mort Toyota Hilux 2005-2015 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C170" s="4" t="inlineStr"/>
-      <c r="D170" s="4" t="inlineStr"/>
+      <c r="C170" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D170" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7238,8 +7914,12 @@
           <t>Unghi mort Lexus ES 2013-2017 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C172" s="4" t="inlineStr"/>
-      <c r="D172" s="4" t="inlineStr"/>
+      <c r="C172" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D172" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7278,8 +7958,12 @@
           <t>Unghi mort Lexus CT 2011-2017 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr"/>
-      <c r="D173" t="inlineStr"/>
+      <c r="C173" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D173" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E173" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7318,8 +8002,12 @@
           <t>Unghi mort Lexus IS 2013-2017 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C174" s="4" t="inlineStr"/>
-      <c r="D174" s="4" t="inlineStr"/>
+      <c r="C174" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D174" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7358,8 +8046,12 @@
           <t>Unghi mort Lexus GS 2012-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr"/>
-      <c r="D175" t="inlineStr"/>
+      <c r="C175" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D175" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E175" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7398,8 +8090,12 @@
           <t>Unghi mort Lexus LS 2013-2017 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C176" s="4" t="inlineStr"/>
-      <c r="D176" s="4" t="inlineStr"/>
+      <c r="C176" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D176" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7438,8 +8134,12 @@
           <t>Unghi mort Lexus NX 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr"/>
-      <c r="D177" t="inlineStr"/>
+      <c r="C177" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D177" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E177" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7478,8 +8178,12 @@
           <t>Unghi mort Lexus RX 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C178" s="4" t="inlineStr"/>
-      <c r="D178" s="4" t="inlineStr"/>
+      <c r="C178" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D178" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7518,8 +8222,12 @@
           <t>Unghi mort Lexus LM 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C179" t="inlineStr"/>
-      <c r="D179" t="inlineStr"/>
+      <c r="C179" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D179" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E179" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7558,8 +8266,12 @@
           <t>Unghi mort Lexus RZ 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C180" s="4" t="inlineStr"/>
-      <c r="D180" s="4" t="inlineStr"/>
+      <c r="C180" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D180" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7598,8 +8310,12 @@
           <t>Unghi mort Lexus RX 2009-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C181" t="inlineStr"/>
-      <c r="D181" t="inlineStr"/>
+      <c r="C181" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D181" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E181" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7638,8 +8354,12 @@
           <t>Unghi mort Lexus LS 2009-2012 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C182" s="4" t="inlineStr"/>
-      <c r="D182" s="4" t="inlineStr"/>
+      <c r="C182" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D182" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7678,8 +8398,12 @@
           <t>Unghi mort Lexus ES 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr"/>
-      <c r="D183" t="inlineStr"/>
+      <c r="C183" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D183" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E183" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7718,8 +8442,12 @@
           <t>Unghi mort Lexus UX 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C184" s="4" t="inlineStr"/>
-      <c r="D184" s="4" t="inlineStr"/>
+      <c r="C184" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D184" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7758,8 +8486,12 @@
           <t>Unghi mort Lexus LC 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr"/>
-      <c r="D185" t="inlineStr"/>
+      <c r="C185" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D185" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E185" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7798,8 +8530,12 @@
           <t>Unghi mort Lexus LS 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C186" s="4" t="inlineStr"/>
-      <c r="D186" s="4" t="inlineStr"/>
+      <c r="C186" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D186" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7838,8 +8574,12 @@
           <t>Unghi mort Lexus GX 2010-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr"/>
-      <c r="D187" t="inlineStr"/>
+      <c r="C187" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D187" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E187" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7878,8 +8618,12 @@
           <t>Unghi mort Lexus ES 2006-2012 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C188" s="4" t="inlineStr"/>
-      <c r="D188" s="4" t="inlineStr"/>
+      <c r="C188" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D188" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7918,8 +8662,12 @@
           <t>Unghi mort Lexus RX 2006-2008 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr"/>
-      <c r="D189" t="inlineStr"/>
+      <c r="C189" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D189" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E189" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -7974,8 +8722,12 @@
           <t>Unghi mort Honda HRV 2015-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr"/>
-      <c r="D191" t="inlineStr"/>
+      <c r="C191" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D191" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E191" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8014,8 +8766,12 @@
           <t>Unghi mort Honda X-RV 2015-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C192" s="4" t="inlineStr"/>
-      <c r="D192" s="4" t="inlineStr"/>
+      <c r="C192" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D192" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8054,8 +8810,12 @@
           <t>Unghi mort Honda Breeze 2020-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr"/>
-      <c r="D193" t="inlineStr"/>
+      <c r="C193" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D193" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E193" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8094,8 +8854,12 @@
           <t>Unghi mort Honda CRV G5 2017-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C194" s="4" t="inlineStr"/>
-      <c r="D194" s="4" t="inlineStr"/>
+      <c r="C194" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D194" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8134,8 +8898,12 @@
           <t>Unghi mort Honda CRV hybrid 2021-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr"/>
-      <c r="D195" t="inlineStr"/>
+      <c r="C195" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D195" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E195" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8174,8 +8942,12 @@
           <t>Unghi mort Honda Crosstour 2010-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C196" s="4" t="inlineStr"/>
-      <c r="D196" s="4" t="inlineStr"/>
+      <c r="C196" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D196" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8214,8 +8986,12 @@
           <t>Unghi mort Honda Honda Fit 2014-2020 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr"/>
-      <c r="D197" t="inlineStr"/>
+      <c r="C197" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D197" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E197" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8254,8 +9030,12 @@
           <t>Unghi mort Honda Honda Jazz 2015-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C198" s="4" t="inlineStr"/>
-      <c r="D198" s="4" t="inlineStr"/>
+      <c r="C198" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D198" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8294,8 +9074,12 @@
           <t>Unghi mort Honda City 2015-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C199" t="inlineStr"/>
-      <c r="D199" t="inlineStr"/>
+      <c r="C199" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D199" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E199" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8334,8 +9118,12 @@
           <t>Unghi mort Honda Honda Fit 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C200" s="4" t="inlineStr"/>
-      <c r="D200" s="4" t="inlineStr"/>
+      <c r="C200" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D200" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8374,8 +9162,12 @@
           <t>Unghi mort Honda Honda Jazz 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C201" t="inlineStr"/>
-      <c r="D201" t="inlineStr"/>
+      <c r="C201" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D201" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E201" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8414,8 +9206,12 @@
           <t>Unghi mort Honda WRV 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C202" s="4" t="inlineStr"/>
-      <c r="D202" s="4" t="inlineStr"/>
+      <c r="C202" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D202" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8454,8 +9250,12 @@
           <t>Unghi mort Honda 2023 BRV  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C203" t="inlineStr"/>
-      <c r="D203" t="inlineStr"/>
+      <c r="C203" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D203" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E203" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8488,8 +9288,12 @@
           <t>Unghi mort Honda Honda Fit 2008-2013 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C204" s="4" t="inlineStr"/>
-      <c r="D204" s="4" t="inlineStr"/>
+      <c r="C204" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D204" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8528,8 +9332,12 @@
           <t>Unghi mort Honda City 2009-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr"/>
-      <c r="D205" t="inlineStr"/>
+      <c r="C205" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D205" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E205" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8568,8 +9376,12 @@
           <t>Unghi mort Honda Honda Civic 10th 2016-2021 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C206" s="4" t="inlineStr"/>
-      <c r="D206" s="4" t="inlineStr"/>
+      <c r="C206" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D206" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8608,8 +9420,12 @@
           <t>Unghi mort Honda ODYSSEY 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C207" t="inlineStr"/>
-      <c r="D207" t="inlineStr"/>
+      <c r="C207" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D207" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E207" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8648,8 +9464,12 @@
           <t>Unghi mort Honda ODYSSEY 2011-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C208" s="4" t="inlineStr"/>
-      <c r="D208" s="4" t="inlineStr"/>
+      <c r="C208" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D208" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8688,8 +9508,12 @@
           <t>Unghi mort Honda Accord 10th ( without right camera) 2018-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C209" t="inlineStr"/>
-      <c r="D209" t="inlineStr"/>
+      <c r="C209" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D209" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E209" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8728,8 +9552,12 @@
           <t>Unghi mort Honda 2024  Accord 11th (without right camera)  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C210" s="4" t="inlineStr"/>
-      <c r="D210" s="4" t="inlineStr"/>
+      <c r="C210" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D210" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8764,8 +9592,12 @@
           <t>Unghi mort Honda Inspire 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C211" t="inlineStr"/>
-      <c r="D211" t="inlineStr"/>
+      <c r="C211" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D211" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E211" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8804,8 +9636,12 @@
           <t>Unghi mort Honda Accord 10th ( with right camera) 2018-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C212" s="4" t="inlineStr"/>
-      <c r="D212" s="4" t="inlineStr"/>
+      <c r="C212" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D212" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8844,8 +9680,12 @@
           <t>Unghi mort Honda 2024  Accord 11th (with right camera)  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C213" t="inlineStr"/>
-      <c r="D213" t="inlineStr"/>
+      <c r="C213" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D213" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E213" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8878,8 +9718,12 @@
           <t>Unghi mort Honda Inspire 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C214" s="4" t="inlineStr"/>
-      <c r="D214" s="4" t="inlineStr"/>
+      <c r="C214" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D214" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8918,8 +9762,12 @@
           <t>Unghi mort Honda Honda Civic 11th 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C215" t="inlineStr"/>
-      <c r="D215" t="inlineStr"/>
+      <c r="C215" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D215" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E215" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8958,8 +9806,12 @@
           <t>Unghi mort Honda HRV 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C216" s="4" t="inlineStr"/>
-      <c r="D216" s="4" t="inlineStr"/>
+      <c r="C216" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D216" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -8998,8 +9850,12 @@
           <t>Unghi mort Honda ZRV 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C217" t="inlineStr"/>
-      <c r="D217" t="inlineStr"/>
+      <c r="C217" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D217" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E217" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9038,8 +9894,12 @@
           <t>Unghi mort Honda e:NP1 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C218" s="4" t="inlineStr"/>
-      <c r="D218" s="4" t="inlineStr"/>
+      <c r="C218" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D218" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9078,8 +9938,12 @@
           <t>Unghi mort Honda CRV 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C219" t="inlineStr"/>
-      <c r="D219" t="inlineStr"/>
+      <c r="C219" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D219" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E219" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9118,8 +9982,12 @@
           <t>Unghi mort Honda XRV 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C220" s="4" t="inlineStr"/>
-      <c r="D220" s="4" t="inlineStr"/>
+      <c r="C220" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D220" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9158,8 +10026,12 @@
           <t>Unghi mort Honda e:NS1 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C221" t="inlineStr"/>
-      <c r="D221" t="inlineStr"/>
+      <c r="C221" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D221" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E221" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9214,8 +10086,12 @@
           <t>Unghi mort Ford Mondeo 2013-2021 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C223" t="inlineStr"/>
-      <c r="D223" t="inlineStr"/>
+      <c r="C223" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D223" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E223" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9254,8 +10130,12 @@
           <t>Unghi mort Ford Mondeo 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C224" s="4" t="inlineStr"/>
-      <c r="D224" s="4" t="inlineStr"/>
+      <c r="C224" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D224" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9294,8 +10174,12 @@
           <t>Unghi mort Ford Mondeo 2008-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C225" t="inlineStr"/>
-      <c r="D225" t="inlineStr"/>
+      <c r="C225" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D225" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E225" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9334,8 +10218,12 @@
           <t>Unghi mort Ford Edge 2015-2020 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C226" s="4" t="inlineStr"/>
-      <c r="D226" s="4" t="inlineStr"/>
+      <c r="C226" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D226" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9374,8 +10262,12 @@
           <t>Unghi mort Ford Edge PLUS 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C227" t="inlineStr"/>
-      <c r="D227" t="inlineStr"/>
+      <c r="C227" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D227" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E227" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9414,8 +10306,12 @@
           <t>Unghi mort Ford Kuga 2013-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C228" s="4" t="inlineStr"/>
-      <c r="D228" s="4" t="inlineStr"/>
+      <c r="C228" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D228" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9454,8 +10350,12 @@
           <t>Unghi mort Ford EcoSport 2013-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C229" t="inlineStr"/>
-      <c r="D229" t="inlineStr"/>
+      <c r="C229" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D229" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E229" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9494,8 +10394,12 @@
           <t>Unghi mort Ford Escape 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C230" s="4" t="inlineStr"/>
-      <c r="D230" s="4" t="inlineStr"/>
+      <c r="C230" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D230" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9534,8 +10438,12 @@
           <t>Unghi mort Ford Escort 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C231" t="inlineStr"/>
-      <c r="D231" t="inlineStr"/>
+      <c r="C231" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D231" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E231" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9574,8 +10482,12 @@
           <t>Unghi mort Ford Explorer 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C232" s="4" t="inlineStr"/>
-      <c r="D232" s="4" t="inlineStr"/>
+      <c r="C232" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D232" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9614,8 +10526,12 @@
           <t>Unghi mort Ford Everest 2016-2020 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C233" t="inlineStr"/>
-      <c r="D233" t="inlineStr"/>
+      <c r="C233" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D233" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E233" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9670,8 +10586,12 @@
           <t>Unghi mort Chevrolet Equinox 2017-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C235" t="inlineStr"/>
-      <c r="D235" t="inlineStr"/>
+      <c r="C235" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D235" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E235" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9710,8 +10630,12 @@
           <t>Unghi mort Chevrolet Malibu 2012-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C236" s="4" t="inlineStr"/>
-      <c r="D236" s="4" t="inlineStr"/>
+      <c r="C236" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D236" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9750,8 +10674,12 @@
           <t>Unghi mort Chevrolet Malibu XL 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C237" t="inlineStr"/>
-      <c r="D237" t="inlineStr"/>
+      <c r="C237" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D237" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E237" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9790,8 +10718,12 @@
           <t>Unghi mort Chevrolet TRAX 2014-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C238" s="4" t="inlineStr"/>
-      <c r="D238" s="4" t="inlineStr"/>
+      <c r="C238" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D238" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9830,8 +10762,12 @@
           <t>Unghi mort Chevrolet TRAX 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C239" t="inlineStr"/>
-      <c r="D239" t="inlineStr"/>
+      <c r="C239" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D239" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E239" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9870,8 +10806,12 @@
           <t>Unghi mort Chevrolet Cruze 2009-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C240" s="4" t="inlineStr"/>
-      <c r="D240" s="4" t="inlineStr"/>
+      <c r="C240" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D240" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9910,8 +10850,12 @@
           <t>Unghi mort Chevrolet Cruze 2015-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C241" t="inlineStr"/>
-      <c r="D241" t="inlineStr"/>
+      <c r="C241" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D241" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E241" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9950,8 +10894,12 @@
           <t>Unghi mort Chevrolet Cruze 2017-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C242" s="4" t="inlineStr"/>
-      <c r="D242" s="4" t="inlineStr"/>
+      <c r="C242" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D242" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -9990,8 +10938,12 @@
           <t>Unghi mort Chevrolet Cruze 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr"/>
-      <c r="D243" t="inlineStr"/>
+      <c r="C243" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D243" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E243" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10030,8 +10982,12 @@
           <t>Unghi mort Chevrolet Cruze 2016-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C244" s="4" t="inlineStr"/>
-      <c r="D244" s="4" t="inlineStr"/>
+      <c r="C244" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D244" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10070,8 +11026,12 @@
           <t>Unghi mort Chevrolet Blazer 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C245" t="inlineStr"/>
-      <c r="D245" t="inlineStr"/>
+      <c r="C245" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D245" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E245" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10110,8 +11070,12 @@
           <t>Unghi mort Chevrolet Orlando 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C246" s="4" t="inlineStr"/>
-      <c r="D246" s="4" t="inlineStr"/>
+      <c r="C246" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D246" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10150,8 +11114,12 @@
           <t>Unghi mort Chevrolet Lova RV 2016-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C247" t="inlineStr"/>
-      <c r="D247" t="inlineStr"/>
+      <c r="C247" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D247" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E247" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10190,8 +11158,12 @@
           <t>Unghi mort Chevrolet Sail 3 2015-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C248" s="4" t="inlineStr"/>
-      <c r="D248" s="4" t="inlineStr"/>
+      <c r="C248" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D248" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10230,8 +11202,12 @@
           <t>Unghi mort Chevrolet AVEO 2011-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C249" t="inlineStr"/>
-      <c r="D249" t="inlineStr"/>
+      <c r="C249" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D249" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E249" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10270,8 +11246,12 @@
           <t>Unghi mort Chevrolet Trailblazer 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C250" s="4" t="inlineStr"/>
-      <c r="D250" s="4" t="inlineStr"/>
+      <c r="C250" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D250" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10310,8 +11290,12 @@
           <t>Unghi mort Chevrolet 2019 Corolado  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C251" t="inlineStr"/>
-      <c r="D251" t="inlineStr"/>
+      <c r="C251" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D251" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E251" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10344,8 +11328,12 @@
           <t>Unghi mort Chevrolet Menlo 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C252" s="4" t="inlineStr"/>
-      <c r="D252" s="4" t="inlineStr"/>
+      <c r="C252" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D252" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10400,8 +11388,12 @@
           <t>Unghi mort Nissan 20212-2025 Patrol Y63 Y62  - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C254" s="4" t="inlineStr"/>
-      <c r="D254" s="4" t="inlineStr"/>
+      <c r="C254" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D254" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10436,8 +11428,12 @@
           <t>Unghi mort Nissan Nissan Sylphy 2012-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C255" t="inlineStr"/>
-      <c r="D255" t="inlineStr"/>
+      <c r="C255" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D255" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E255" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10476,8 +11472,12 @@
           <t>Unghi mort Nissan Nissan Altima 2013-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C256" s="4" t="inlineStr"/>
-      <c r="D256" s="4" t="inlineStr"/>
+      <c r="C256" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D256" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10516,8 +11516,12 @@
           <t>Unghi mort Nissan Nissan TIIDA 2016-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C257" t="inlineStr"/>
-      <c r="D257" t="inlineStr"/>
+      <c r="C257" s="29" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D257" s="30" t="n">
+        <v>1100</v>
+      </c>
       <c r="E257" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10556,8 +11560,12 @@
           <t>Unghi mort Nissan Altima 2019-2025 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C258" s="4" t="inlineStr"/>
-      <c r="D258" s="4" t="inlineStr"/>
+      <c r="C258" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D258" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10596,8 +11604,12 @@
           <t>Unghi mort Nissan Qashqai 2016-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C259" t="inlineStr"/>
-      <c r="D259" t="inlineStr"/>
+      <c r="C259" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D259" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E259" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10636,8 +11648,12 @@
           <t>Unghi mort Nissan Murano 2015-2025 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C260" s="4" t="inlineStr"/>
-      <c r="D260" s="4" t="inlineStr"/>
+      <c r="C260" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D260" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10676,8 +11692,12 @@
           <t>Unghi mort Nissan Nissan X-Trail 2022-2025 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C261" t="inlineStr"/>
-      <c r="D261" t="inlineStr"/>
+      <c r="C261" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D261" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E261" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10716,8 +11736,12 @@
           <t>Unghi mort Nissan Nissan X-Trail 2014-2021 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C262" s="4" t="inlineStr"/>
-      <c r="D262" s="4" t="inlineStr"/>
+      <c r="C262" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D262" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E262" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10772,8 +11796,12 @@
           <t>Unghi mort Mazda Mazda 3 2014-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C264" s="4" t="inlineStr"/>
-      <c r="D264" s="4" t="inlineStr"/>
+      <c r="C264" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D264" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E264" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10812,8 +11840,12 @@
           <t>Unghi mort Mazda Mazda 3 2017-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C265" t="inlineStr"/>
-      <c r="D265" t="inlineStr"/>
+      <c r="C265" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D265" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E265" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10852,8 +11884,12 @@
           <t>Unghi mort Mazda Mazda 6 2014-2021 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C266" s="4" t="inlineStr"/>
-      <c r="D266" s="4" t="inlineStr"/>
+      <c r="C266" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D266" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10892,8 +11928,12 @@
           <t>Unghi mort Mazda CX4 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C267" t="inlineStr"/>
-      <c r="D267" t="inlineStr"/>
+      <c r="C267" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D267" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E267" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10932,8 +11972,12 @@
           <t>Unghi mort Mazda CX5 2015-2017 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C268" s="4" t="inlineStr"/>
-      <c r="D268" s="4" t="inlineStr"/>
+      <c r="C268" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D268" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -10972,8 +12016,12 @@
           <t>Unghi mort Mazda CX5 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C269" t="inlineStr"/>
-      <c r="D269" t="inlineStr"/>
+      <c r="C269" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D269" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E269" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11012,8 +12060,12 @@
           <t>Unghi mort Mazda CX3 2016-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C270" s="4" t="inlineStr"/>
-      <c r="D270" s="4" t="inlineStr"/>
+      <c r="C270" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D270" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11052,8 +12104,12 @@
           <t>Unghi mort Mazda CX8 2018-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C271" t="inlineStr"/>
-      <c r="D271" t="inlineStr"/>
+      <c r="C271" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D271" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E271" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11092,8 +12148,12 @@
           <t>Unghi mort Mazda Mazda 3 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C272" s="4" t="inlineStr"/>
-      <c r="D272" s="4" t="inlineStr"/>
+      <c r="C272" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D272" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11132,8 +12192,12 @@
           <t>Unghi mort Mazda Mazda Axela 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C273" t="inlineStr"/>
-      <c r="D273" t="inlineStr"/>
+      <c r="C273" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D273" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E273" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11172,8 +12236,12 @@
           <t>Unghi mort Mazda Mazda 2 2007-2012 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C274" s="4" t="inlineStr"/>
-      <c r="D274" s="4" t="inlineStr"/>
+      <c r="C274" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D274" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11212,8 +12280,12 @@
           <t>Unghi mort Mazda Mazda 3 2011-2013 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C275" t="inlineStr"/>
-      <c r="D275" t="inlineStr"/>
+      <c r="C275" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D275" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E275" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11252,8 +12324,12 @@
           <t>Unghi mort Mazda Mazda 6 2009-2015 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C276" s="4" t="inlineStr"/>
-      <c r="D276" s="4" t="inlineStr"/>
+      <c r="C276" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D276" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11292,8 +12368,12 @@
           <t>Unghi mort Mazda Mazda CX30 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C277" t="inlineStr"/>
-      <c r="D277" t="inlineStr"/>
+      <c r="C277" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D277" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E277" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11348,8 +12428,12 @@
           <t>Unghi mort Porsche Panamera 2009-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C279" t="inlineStr"/>
-      <c r="D279" t="inlineStr"/>
+      <c r="C279" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D279" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E279" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11388,8 +12472,12 @@
           <t>Unghi mort Porsche Cayenne 2011-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C280" s="4" t="inlineStr"/>
-      <c r="D280" s="4" t="inlineStr"/>
+      <c r="C280" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D280" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E280" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11428,8 +12516,12 @@
           <t>Unghi mort Porsche Cayenne 2015-2017 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C281" t="inlineStr"/>
-      <c r="D281" t="inlineStr"/>
+      <c r="C281" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D281" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E281" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11468,8 +12560,12 @@
           <t>Unghi mort Porsche Panamera 2017-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C282" s="4" t="inlineStr"/>
-      <c r="D282" s="4" t="inlineStr"/>
+      <c r="C282" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D282" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11508,8 +12604,12 @@
           <t>Unghi mort Porsche Cayenne 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C283" t="inlineStr"/>
-      <c r="D283" t="inlineStr"/>
+      <c r="C283" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D283" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E283" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11548,8 +12648,12 @@
           <t>Unghi mort Porsche 718/Boxster 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C284" s="4" t="inlineStr"/>
-      <c r="D284" s="4" t="inlineStr"/>
+      <c r="C284" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D284" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E284" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11588,8 +12692,12 @@
           <t>Unghi mort Porsche Macan 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C285" t="inlineStr"/>
-      <c r="D285" t="inlineStr"/>
+      <c r="C285" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D285" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E285" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11628,8 +12736,12 @@
           <t>Unghi mort Porsche Taycan 2019-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C286" s="4" t="inlineStr"/>
-      <c r="D286" s="4" t="inlineStr"/>
+      <c r="C286" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D286" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11668,8 +12780,12 @@
           <t>Unghi mort Porsche 911 2020-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C287" t="inlineStr"/>
-      <c r="D287" t="inlineStr"/>
+      <c r="C287" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D287" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E287" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11724,8 +12840,12 @@
           <t>Unghi mort Land Rover Freelander 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C289" t="inlineStr"/>
-      <c r="D289" t="inlineStr"/>
+      <c r="C289" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D289" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E289" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11764,8 +12884,12 @@
           <t>Unghi mort Land Rover Range Rover Evoque 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C290" s="4" t="inlineStr"/>
-      <c r="D290" s="4" t="inlineStr"/>
+      <c r="C290" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D290" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11804,8 +12928,12 @@
           <t>Unghi mort Land Rover Range Rover 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C291" t="inlineStr"/>
-      <c r="D291" t="inlineStr"/>
+      <c r="C291" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D291" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E291" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11844,8 +12972,12 @@
           <t>Unghi mort Land Rover Range Rover sport 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C292" s="4" t="inlineStr"/>
-      <c r="D292" s="4" t="inlineStr"/>
+      <c r="C292" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D292" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11884,8 +13016,12 @@
           <t>Unghi mort Land Rover Discover 4 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C293" t="inlineStr"/>
-      <c r="D293" t="inlineStr"/>
+      <c r="C293" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D293" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E293" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11924,8 +13060,12 @@
           <t>Unghi mort Land Rover Discover 5 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C294" s="4" t="inlineStr"/>
-      <c r="D294" s="4" t="inlineStr"/>
+      <c r="C294" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D294" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -11964,8 +13104,12 @@
           <t>Unghi mort Land Rover Freelander 2 2010-2015 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C295" t="inlineStr"/>
-      <c r="D295" t="inlineStr"/>
+      <c r="C295" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D295" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E295" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12004,8 +13148,12 @@
           <t>Unghi mort Land Rover Discover 4 2010-2013 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C296" s="4" t="inlineStr"/>
-      <c r="D296" s="4" t="inlineStr"/>
+      <c r="C296" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D296" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12044,8 +13192,12 @@
           <t>Unghi mort Land Rover Range Rover Evoque 2011-2013 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C297" t="inlineStr"/>
-      <c r="D297" t="inlineStr"/>
+      <c r="C297" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D297" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E297" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12084,8 +13236,12 @@
           <t>Unghi mort Land Rover Discover 3 2005-2009 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C298" s="4" t="inlineStr"/>
-      <c r="D298" s="4" t="inlineStr"/>
+      <c r="C298" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D298" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E298" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12124,8 +13280,12 @@
           <t>Unghi mort Land Rover Freelander 2 2007-2009 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C299" t="inlineStr"/>
-      <c r="D299" t="inlineStr"/>
+      <c r="C299" s="29" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D299" s="30" t="n">
+        <v>1200</v>
+      </c>
       <c r="E299" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12164,8 +13324,12 @@
           <t>Unghi mort Land Rover Range Rover 2005-2008 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C300" s="4" t="inlineStr"/>
-      <c r="D300" s="4" t="inlineStr"/>
+      <c r="C300" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D300" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12204,8 +13368,12 @@
           <t>Unghi mort Land Rover Range Rover sport 2005-2009 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C301" t="inlineStr"/>
-      <c r="D301" t="inlineStr"/>
+      <c r="C301" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D301" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E301" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12260,8 +13428,12 @@
           <t>Unghi mort Maserati Ghibli 2014-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C303" t="inlineStr"/>
-      <c r="D303" t="inlineStr"/>
+      <c r="C303" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D303" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E303" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12300,8 +13472,12 @@
           <t>Unghi mort Maserati Quattroporte 2014-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C304" s="4" t="inlineStr"/>
-      <c r="D304" s="4" t="inlineStr"/>
+      <c r="C304" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D304" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12340,8 +13516,12 @@
           <t>Unghi mort Maserati Ghibli 2017-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C305" t="inlineStr"/>
-      <c r="D305" t="inlineStr"/>
+      <c r="C305" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D305" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E305" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12380,8 +13560,12 @@
           <t>Unghi mort Maserati Quattroporte 2017-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C306" s="4" t="inlineStr"/>
-      <c r="D306" s="4" t="inlineStr"/>
+      <c r="C306" s="29" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D306" s="30" t="n">
+        <v>1450</v>
+      </c>
       <c r="E306" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12420,8 +13604,12 @@
           <t>Unghi mort Maserati Levante 2016-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C307" t="inlineStr"/>
-      <c r="D307" t="inlineStr"/>
+      <c r="C307" s="29" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D307" s="30" t="n">
+        <v>1600</v>
+      </c>
       <c r="E307" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12476,8 +13664,12 @@
           <t>Unghi mort Chery Tiggo 8 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C309" t="inlineStr"/>
-      <c r="D309" t="inlineStr"/>
+      <c r="C309" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D309" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E309" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12516,8 +13708,12 @@
           <t>Unghi mort Chery Tiggo 8 PLUS 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C310" s="4" t="inlineStr"/>
-      <c r="D310" s="4" t="inlineStr"/>
+      <c r="C310" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D310" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12556,8 +13752,12 @@
           <t>Unghi mort Chery Tiggo 7 2020-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C311" t="inlineStr"/>
-      <c r="D311" t="inlineStr"/>
+      <c r="C311" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D311" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E311" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12596,8 +13796,12 @@
           <t>Unghi mort Chery Tiggo E 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C312" s="4" t="inlineStr"/>
-      <c r="D312" s="4" t="inlineStr"/>
+      <c r="C312" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D312" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12636,8 +13840,12 @@
           <t>Unghi mort Chery Tiggo 8 pro 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C313" t="inlineStr"/>
-      <c r="D313" t="inlineStr"/>
+      <c r="C313" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D313" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E313" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12676,8 +13884,12 @@
           <t>Unghi mort Chery Tiggo 7 plus 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C314" s="4" t="inlineStr"/>
-      <c r="D314" s="4" t="inlineStr"/>
+      <c r="C314" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D314" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
           <t>BSD-01</t>
@@ -12716,8 +13928,12 @@
           <t>Unghi mort Chery Tiggo 9 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
-      <c r="C315" t="inlineStr"/>
-      <c r="D315" t="inlineStr"/>
+      <c r="C315" s="29" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D315" s="30" t="n">
+        <v>1300</v>
+      </c>
       <c r="E315" t="inlineStr">
         <is>
           <t>BSD-01</t>

</xml_diff>

<commit_message>
BSD-Catalog-Master - dealer price -25%
</commit_message>
<xml_diff>
--- a/BSD-Catalog-Master.xlsx
+++ b/BSD-Catalog-Master.xlsx
@@ -632,7 +632,7 @@
         <v>1199</v>
       </c>
       <c r="D3" s="30" t="n">
-        <v>950</v>
+        <v>900</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
         <v>1399</v>
       </c>
       <c r="D4" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
@@ -720,7 +720,7 @@
         <v>1399</v>
       </c>
       <c r="D5" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
         <v>1399</v>
       </c>
       <c r="D6" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
@@ -808,7 +808,7 @@
         <v>1399</v>
       </c>
       <c r="D7" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -852,7 +852,7 @@
         <v>1199</v>
       </c>
       <c r="D8" s="30" t="n">
-        <v>950</v>
+        <v>900</v>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
         <v>1399</v>
       </c>
       <c r="D9" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
         <v>1399</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
@@ -984,7 +984,7 @@
         <v>1399</v>
       </c>
       <c r="D11" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1028,7 +1028,7 @@
         <v>1399</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
@@ -1072,7 +1072,7 @@
         <v>1499</v>
       </c>
       <c r="D13" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1116,7 +1116,7 @@
         <v>1599</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
@@ -1160,7 +1160,7 @@
         <v>1499</v>
       </c>
       <c r="D15" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1204,7 +1204,7 @@
         <v>1399</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
         <v>1799</v>
       </c>
       <c r="D17" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1292,7 +1292,7 @@
         <v>1599</v>
       </c>
       <c r="D18" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
@@ -1336,7 +1336,7 @@
         <v>1799</v>
       </c>
       <c r="D19" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1380,7 +1380,7 @@
         <v>1799</v>
       </c>
       <c r="D20" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
         <v>1799</v>
       </c>
       <c r="D21" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1468,7 +1468,7 @@
         <v>1799</v>
       </c>
       <c r="D22" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
@@ -1512,7 +1512,7 @@
         <v>1599</v>
       </c>
       <c r="D23" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1556,7 +1556,7 @@
         <v>1799</v>
       </c>
       <c r="D24" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
@@ -1600,7 +1600,7 @@
         <v>1799</v>
       </c>
       <c r="D25" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1644,7 +1644,7 @@
         <v>1999</v>
       </c>
       <c r="D26" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
@@ -1688,7 +1688,7 @@
         <v>1499</v>
       </c>
       <c r="D27" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1732,7 +1732,7 @@
         <v>1999</v>
       </c>
       <c r="D28" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
@@ -1776,7 +1776,7 @@
         <v>1999</v>
       </c>
       <c r="D29" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1820,7 +1820,7 @@
         <v>1799</v>
       </c>
       <c r="D30" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
@@ -1864,7 +1864,7 @@
         <v>1799</v>
       </c>
       <c r="D31" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
         <v>1799</v>
       </c>
       <c r="D32" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
@@ -1952,7 +1952,7 @@
         <v>1999</v>
       </c>
       <c r="D33" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1996,7 +1996,7 @@
         <v>1999</v>
       </c>
       <c r="D34" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
@@ -2040,7 +2040,7 @@
         <v>1799</v>
       </c>
       <c r="D35" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2084,7 +2084,7 @@
         <v>1999</v>
       </c>
       <c r="D36" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v>1999</v>
       </c>
       <c r="D37" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -2172,7 +2172,7 @@
         <v>1999</v>
       </c>
       <c r="D38" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
@@ -2216,7 +2216,7 @@
         <v>1999</v>
       </c>
       <c r="D39" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -2260,7 +2260,7 @@
         <v>1999</v>
       </c>
       <c r="D40" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
@@ -2304,7 +2304,7 @@
         <v>1999</v>
       </c>
       <c r="D41" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
         <v>1999</v>
       </c>
       <c r="D42" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
@@ -2392,7 +2392,7 @@
         <v>1999</v>
       </c>
       <c r="D43" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         <v>1999</v>
       </c>
       <c r="D44" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
@@ -2480,7 +2480,7 @@
         <v>1999</v>
       </c>
       <c r="D45" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2540,7 +2540,7 @@
         <v>1599</v>
       </c>
       <c r="D47" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         <v>1999</v>
       </c>
       <c r="D48" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
@@ -2628,7 +2628,7 @@
         <v>1599</v>
       </c>
       <c r="D49" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -2672,7 +2672,7 @@
         <v>1599</v>
       </c>
       <c r="D50" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
@@ -2716,7 +2716,7 @@
         <v>1599</v>
       </c>
       <c r="D51" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -2760,7 +2760,7 @@
         <v>1999</v>
       </c>
       <c r="D52" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
         <v>1999</v>
       </c>
       <c r="D53" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
         <v>1599</v>
       </c>
       <c r="D54" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
@@ -2892,7 +2892,7 @@
         <v>1799</v>
       </c>
       <c r="D55" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2936,7 +2936,7 @@
         <v>1999</v>
       </c>
       <c r="D56" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
@@ -2980,7 +2980,7 @@
         <v>1399</v>
       </c>
       <c r="D57" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -3024,7 +3024,7 @@
         <v>1499</v>
       </c>
       <c r="D58" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
@@ -3068,7 +3068,7 @@
         <v>1599</v>
       </c>
       <c r="D59" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -3112,7 +3112,7 @@
         <v>1499</v>
       </c>
       <c r="D60" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
@@ -3156,7 +3156,7 @@
         <v>1799</v>
       </c>
       <c r="D61" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -3200,7 +3200,7 @@
         <v>1499</v>
       </c>
       <c r="D62" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
@@ -3244,7 +3244,7 @@
         <v>1499</v>
       </c>
       <c r="D63" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -3288,7 +3288,7 @@
         <v>1499</v>
       </c>
       <c r="D64" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
@@ -3332,7 +3332,7 @@
         <v>1499</v>
       </c>
       <c r="D65" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3376,7 +3376,7 @@
         <v>1799</v>
       </c>
       <c r="D66" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
@@ -3420,7 +3420,7 @@
         <v>1399</v>
       </c>
       <c r="D67" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -3464,7 +3464,7 @@
         <v>1999</v>
       </c>
       <c r="D68" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
@@ -3508,7 +3508,7 @@
         <v>1599</v>
       </c>
       <c r="D69" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -3552,7 +3552,7 @@
         <v>1599</v>
       </c>
       <c r="D70" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
@@ -3596,7 +3596,7 @@
         <v>1799</v>
       </c>
       <c r="D71" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -3640,7 +3640,7 @@
         <v>1999</v>
       </c>
       <c r="D72" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
@@ -3684,7 +3684,7 @@
         <v>1799</v>
       </c>
       <c r="D73" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -3728,7 +3728,7 @@
         <v>1599</v>
       </c>
       <c r="D74" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
@@ -3772,7 +3772,7 @@
         <v>1599</v>
       </c>
       <c r="D75" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3816,7 +3816,7 @@
         <v>1799</v>
       </c>
       <c r="D76" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
@@ -3860,7 +3860,7 @@
         <v>1999</v>
       </c>
       <c r="D77" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -3904,7 +3904,7 @@
         <v>1999</v>
       </c>
       <c r="D78" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
         <v>1799</v>
       </c>
       <c r="D79" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -3992,7 +3992,7 @@
         <v>1999</v>
       </c>
       <c r="D80" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
         <v>1999</v>
       </c>
       <c r="D81" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -4080,7 +4080,7 @@
         <v>1399</v>
       </c>
       <c r="D82" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
@@ -4124,7 +4124,7 @@
         <v>1399</v>
       </c>
       <c r="D83" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -4168,7 +4168,7 @@
         <v>1399</v>
       </c>
       <c r="D84" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
@@ -4212,7 +4212,7 @@
         <v>1999</v>
       </c>
       <c r="D85" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -4256,7 +4256,7 @@
         <v>1799</v>
       </c>
       <c r="D86" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
@@ -4300,7 +4300,7 @@
         <v>1999</v>
       </c>
       <c r="D87" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -4344,7 +4344,7 @@
         <v>1999</v>
       </c>
       <c r="D88" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
@@ -4388,7 +4388,7 @@
         <v>1999</v>
       </c>
       <c r="D89" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -4432,7 +4432,7 @@
         <v>1799</v>
       </c>
       <c r="D90" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
@@ -4476,7 +4476,7 @@
         <v>1999</v>
       </c>
       <c r="D91" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -4536,7 +4536,7 @@
         <v>1499</v>
       </c>
       <c r="D93" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -4580,7 +4580,7 @@
         <v>1799</v>
       </c>
       <c r="D94" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
@@ -4624,7 +4624,7 @@
         <v>1499</v>
       </c>
       <c r="D95" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -4668,7 +4668,7 @@
         <v>1799</v>
       </c>
       <c r="D96" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
@@ -4712,7 +4712,7 @@
         <v>1399</v>
       </c>
       <c r="D97" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -4756,7 +4756,7 @@
         <v>1599</v>
       </c>
       <c r="D98" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
@@ -4800,7 +4800,7 @@
         <v>1599</v>
       </c>
       <c r="D99" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -4844,7 +4844,7 @@
         <v>1599</v>
       </c>
       <c r="D100" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
@@ -4888,7 +4888,7 @@
         <v>1599</v>
       </c>
       <c r="D101" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -4932,7 +4932,7 @@
         <v>1499</v>
       </c>
       <c r="D102" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
@@ -4976,7 +4976,7 @@
         <v>1599</v>
       </c>
       <c r="D103" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -5020,7 +5020,7 @@
         <v>1599</v>
       </c>
       <c r="D104" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
@@ -5064,7 +5064,7 @@
         <v>1799</v>
       </c>
       <c r="D105" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -5108,7 +5108,7 @@
         <v>1399</v>
       </c>
       <c r="D106" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
         <v>1799</v>
       </c>
       <c r="D107" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -5192,7 +5192,7 @@
         <v>1799</v>
       </c>
       <c r="D108" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
@@ -5236,7 +5236,7 @@
         <v>1999</v>
       </c>
       <c r="D109" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -5280,7 +5280,7 @@
         <v>1999</v>
       </c>
       <c r="D110" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
@@ -5324,7 +5324,7 @@
         <v>1999</v>
       </c>
       <c r="D111" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -5368,7 +5368,7 @@
         <v>1799</v>
       </c>
       <c r="D112" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
@@ -5412,7 +5412,7 @@
         <v>1799</v>
       </c>
       <c r="D113" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -5456,7 +5456,7 @@
         <v>1799</v>
       </c>
       <c r="D114" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
@@ -5500,7 +5500,7 @@
         <v>1999</v>
       </c>
       <c r="D115" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -5544,7 +5544,7 @@
         <v>1999</v>
       </c>
       <c r="D116" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
@@ -5588,7 +5588,7 @@
         <v>1999</v>
       </c>
       <c r="D117" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -5632,7 +5632,7 @@
         <v>1599</v>
       </c>
       <c r="D118" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
@@ -5676,7 +5676,7 @@
         <v>1799</v>
       </c>
       <c r="D119" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -5720,7 +5720,7 @@
         <v>1799</v>
       </c>
       <c r="D120" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
@@ -5764,7 +5764,7 @@
         <v>1599</v>
       </c>
       <c r="D121" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -5808,7 +5808,7 @@
         <v>1999</v>
       </c>
       <c r="D122" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
@@ -5852,7 +5852,7 @@
         <v>1599</v>
       </c>
       <c r="D123" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -5896,7 +5896,7 @@
         <v>1999</v>
       </c>
       <c r="D124" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
@@ -5940,7 +5940,7 @@
         <v>1599</v>
       </c>
       <c r="D125" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -5984,7 +5984,7 @@
         <v>1999</v>
       </c>
       <c r="D126" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
@@ -6028,7 +6028,7 @@
         <v>1999</v>
       </c>
       <c r="D127" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -6072,7 +6072,7 @@
         <v>1999</v>
       </c>
       <c r="D128" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
@@ -6112,7 +6112,7 @@
         <v>1999</v>
       </c>
       <c r="D129" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v>1399</v>
       </c>
       <c r="D130" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
@@ -6200,7 +6200,7 @@
         <v>1599</v>
       </c>
       <c r="D131" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -6244,7 +6244,7 @@
         <v>1599</v>
       </c>
       <c r="D132" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
@@ -6288,7 +6288,7 @@
         <v>1799</v>
       </c>
       <c r="D133" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -6326,7 +6326,7 @@
         <v>1499</v>
       </c>
       <c r="D134" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
@@ -6366,7 +6366,7 @@
         <v>1499</v>
       </c>
       <c r="D135" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -6404,7 +6404,7 @@
         <v>1999</v>
       </c>
       <c r="D136" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
@@ -6448,7 +6448,7 @@
         <v>1799</v>
       </c>
       <c r="D137" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -6492,7 +6492,7 @@
         <v>1999</v>
       </c>
       <c r="D138" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
@@ -6532,7 +6532,7 @@
         <v>1799</v>
       </c>
       <c r="D139" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -6576,7 +6576,7 @@
         <v>1399</v>
       </c>
       <c r="D140" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
@@ -6632,7 +6632,7 @@
         <v>1799</v>
       </c>
       <c r="D142" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
@@ -6676,7 +6676,7 @@
         <v>1599</v>
       </c>
       <c r="D143" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -6720,7 +6720,7 @@
         <v>1799</v>
       </c>
       <c r="D144" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
@@ -6764,7 +6764,7 @@
         <v>1799</v>
       </c>
       <c r="D145" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -6808,7 +6808,7 @@
         <v>1799</v>
       </c>
       <c r="D146" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
@@ -6852,7 +6852,7 @@
         <v>1599</v>
       </c>
       <c r="D147" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -6896,7 +6896,7 @@
         <v>1599</v>
       </c>
       <c r="D148" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
@@ -6940,7 +6940,7 @@
         <v>1999</v>
       </c>
       <c r="D149" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -6984,7 +6984,7 @@
         <v>1599</v>
       </c>
       <c r="D150" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
@@ -7028,7 +7028,7 @@
         <v>1599</v>
       </c>
       <c r="D151" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -7072,7 +7072,7 @@
         <v>1599</v>
       </c>
       <c r="D152" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
@@ -7116,7 +7116,7 @@
         <v>1599</v>
       </c>
       <c r="D153" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -7160,7 +7160,7 @@
         <v>1599</v>
       </c>
       <c r="D154" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
@@ -7204,7 +7204,7 @@
         <v>1999</v>
       </c>
       <c r="D155" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -7248,7 +7248,7 @@
         <v>1999</v>
       </c>
       <c r="D156" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
@@ -7292,7 +7292,7 @@
         <v>1199</v>
       </c>
       <c r="D157" s="30" t="n">
-        <v>950</v>
+        <v>900</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -7336,7 +7336,7 @@
         <v>1499</v>
       </c>
       <c r="D158" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
@@ -7380,7 +7380,7 @@
         <v>1599</v>
       </c>
       <c r="D159" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -7424,7 +7424,7 @@
         <v>1599</v>
       </c>
       <c r="D160" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
@@ -7468,7 +7468,7 @@
         <v>1999</v>
       </c>
       <c r="D161" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -7512,7 +7512,7 @@
         <v>1999</v>
       </c>
       <c r="D162" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
@@ -7556,7 +7556,7 @@
         <v>1399</v>
       </c>
       <c r="D163" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -7600,7 +7600,7 @@
         <v>1499</v>
       </c>
       <c r="D164" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
@@ -7644,7 +7644,7 @@
         <v>1499</v>
       </c>
       <c r="D165" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -7688,7 +7688,7 @@
         <v>1499</v>
       </c>
       <c r="D166" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
@@ -7732,7 +7732,7 @@
         <v>1399</v>
       </c>
       <c r="D167" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -7776,7 +7776,7 @@
         <v>1499</v>
       </c>
       <c r="D168" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
@@ -7820,7 +7820,7 @@
         <v>1499</v>
       </c>
       <c r="D169" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
         <v>1499</v>
       </c>
       <c r="D170" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
@@ -7918,7 +7918,7 @@
         <v>1599</v>
       </c>
       <c r="D172" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
@@ -7962,7 +7962,7 @@
         <v>1399</v>
       </c>
       <c r="D173" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -8006,7 +8006,7 @@
         <v>1499</v>
       </c>
       <c r="D174" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
@@ -8050,7 +8050,7 @@
         <v>1499</v>
       </c>
       <c r="D175" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -8094,7 +8094,7 @@
         <v>1999</v>
       </c>
       <c r="D176" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
@@ -8138,7 +8138,7 @@
         <v>1799</v>
       </c>
       <c r="D177" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -8182,7 +8182,7 @@
         <v>1999</v>
       </c>
       <c r="D178" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
@@ -8226,7 +8226,7 @@
         <v>1799</v>
       </c>
       <c r="D179" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -8270,7 +8270,7 @@
         <v>1799</v>
       </c>
       <c r="D180" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
@@ -8314,7 +8314,7 @@
         <v>1799</v>
       </c>
       <c r="D181" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -8358,7 +8358,7 @@
         <v>1999</v>
       </c>
       <c r="D182" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
@@ -8402,7 +8402,7 @@
         <v>1799</v>
       </c>
       <c r="D183" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -8446,7 +8446,7 @@
         <v>1799</v>
       </c>
       <c r="D184" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
@@ -8490,7 +8490,7 @@
         <v>1999</v>
       </c>
       <c r="D185" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -8534,7 +8534,7 @@
         <v>1999</v>
       </c>
       <c r="D186" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
@@ -8578,7 +8578,7 @@
         <v>1999</v>
       </c>
       <c r="D187" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -8622,7 +8622,7 @@
         <v>1599</v>
       </c>
       <c r="D188" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
@@ -8666,7 +8666,7 @@
         <v>1799</v>
       </c>
       <c r="D189" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -8726,7 +8726,7 @@
         <v>1599</v>
       </c>
       <c r="D191" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -8770,7 +8770,7 @@
         <v>1599</v>
       </c>
       <c r="D192" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
@@ -8814,7 +8814,7 @@
         <v>1799</v>
       </c>
       <c r="D193" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -8858,7 +8858,7 @@
         <v>1799</v>
       </c>
       <c r="D194" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
@@ -8902,7 +8902,7 @@
         <v>1799</v>
       </c>
       <c r="D195" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -8946,7 +8946,7 @@
         <v>1499</v>
       </c>
       <c r="D196" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
@@ -8990,7 +8990,7 @@
         <v>1499</v>
       </c>
       <c r="D197" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -9034,7 +9034,7 @@
         <v>1499</v>
       </c>
       <c r="D198" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
@@ -9078,7 +9078,7 @@
         <v>1499</v>
       </c>
       <c r="D199" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -9122,7 +9122,7 @@
         <v>1599</v>
       </c>
       <c r="D200" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
@@ -9166,7 +9166,7 @@
         <v>1599</v>
       </c>
       <c r="D201" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -9210,7 +9210,7 @@
         <v>1599</v>
       </c>
       <c r="D202" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
@@ -9254,7 +9254,7 @@
         <v>1499</v>
       </c>
       <c r="D203" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -9292,7 +9292,7 @@
         <v>1499</v>
       </c>
       <c r="D204" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
@@ -9336,7 +9336,7 @@
         <v>1499</v>
       </c>
       <c r="D205" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -9380,7 +9380,7 @@
         <v>1599</v>
       </c>
       <c r="D206" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
@@ -9424,7 +9424,7 @@
         <v>1799</v>
       </c>
       <c r="D207" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -9468,7 +9468,7 @@
         <v>1599</v>
       </c>
       <c r="D208" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
@@ -9512,7 +9512,7 @@
         <v>1799</v>
       </c>
       <c r="D209" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -9556,7 +9556,7 @@
         <v>1499</v>
       </c>
       <c r="D210" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
@@ -9596,7 +9596,7 @@
         <v>1599</v>
       </c>
       <c r="D211" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -9640,7 +9640,7 @@
         <v>1799</v>
       </c>
       <c r="D212" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
@@ -9684,7 +9684,7 @@
         <v>1499</v>
       </c>
       <c r="D213" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -9722,7 +9722,7 @@
         <v>1599</v>
       </c>
       <c r="D214" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
@@ -9766,7 +9766,7 @@
         <v>1599</v>
       </c>
       <c r="D215" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -9810,7 +9810,7 @@
         <v>1599</v>
       </c>
       <c r="D216" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
@@ -9854,7 +9854,7 @@
         <v>1799</v>
       </c>
       <c r="D217" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -9898,7 +9898,7 @@
         <v>1599</v>
       </c>
       <c r="D218" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
@@ -9942,7 +9942,7 @@
         <v>1799</v>
       </c>
       <c r="D219" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -9986,7 +9986,7 @@
         <v>1599</v>
       </c>
       <c r="D220" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
@@ -10030,7 +10030,7 @@
         <v>1599</v>
       </c>
       <c r="D221" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -10090,7 +10090,7 @@
         <v>1399</v>
       </c>
       <c r="D223" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -10134,7 +10134,7 @@
         <v>1399</v>
       </c>
       <c r="D224" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
@@ -10178,7 +10178,7 @@
         <v>1399</v>
       </c>
       <c r="D225" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -10222,7 +10222,7 @@
         <v>1499</v>
       </c>
       <c r="D226" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
@@ -10266,7 +10266,7 @@
         <v>1799</v>
       </c>
       <c r="D227" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -10310,7 +10310,7 @@
         <v>1499</v>
       </c>
       <c r="D228" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
@@ -10354,7 +10354,7 @@
         <v>1499</v>
       </c>
       <c r="D229" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -10398,7 +10398,7 @@
         <v>1599</v>
       </c>
       <c r="D230" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
@@ -10442,7 +10442,7 @@
         <v>1599</v>
       </c>
       <c r="D231" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -10486,7 +10486,7 @@
         <v>1999</v>
       </c>
       <c r="D232" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
@@ -10530,7 +10530,7 @@
         <v>1499</v>
       </c>
       <c r="D233" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -10590,7 +10590,7 @@
         <v>1599</v>
       </c>
       <c r="D235" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -10634,7 +10634,7 @@
         <v>1399</v>
       </c>
       <c r="D236" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
@@ -10678,7 +10678,7 @@
         <v>1599</v>
       </c>
       <c r="D237" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -10722,7 +10722,7 @@
         <v>1399</v>
       </c>
       <c r="D238" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
@@ -10766,7 +10766,7 @@
         <v>1599</v>
       </c>
       <c r="D239" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -10810,7 +10810,7 @@
         <v>1499</v>
       </c>
       <c r="D240" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
@@ -10854,7 +10854,7 @@
         <v>1499</v>
       </c>
       <c r="D241" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -10898,7 +10898,7 @@
         <v>1499</v>
       </c>
       <c r="D242" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
@@ -10942,7 +10942,7 @@
         <v>1599</v>
       </c>
       <c r="D243" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -10986,7 +10986,7 @@
         <v>1499</v>
       </c>
       <c r="D244" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
@@ -11030,7 +11030,7 @@
         <v>1799</v>
       </c>
       <c r="D245" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -11074,7 +11074,7 @@
         <v>1599</v>
       </c>
       <c r="D246" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
@@ -11118,7 +11118,7 @@
         <v>1499</v>
       </c>
       <c r="D247" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -11162,7 +11162,7 @@
         <v>1499</v>
       </c>
       <c r="D248" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
@@ -11206,7 +11206,7 @@
         <v>1499</v>
       </c>
       <c r="D249" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -11250,7 +11250,7 @@
         <v>1599</v>
       </c>
       <c r="D250" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
@@ -11294,7 +11294,7 @@
         <v>1499</v>
       </c>
       <c r="D251" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -11332,7 +11332,7 @@
         <v>1599</v>
       </c>
       <c r="D252" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
@@ -11392,7 +11392,7 @@
         <v>1799</v>
       </c>
       <c r="D254" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
@@ -11432,7 +11432,7 @@
         <v>1399</v>
       </c>
       <c r="D255" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -11476,7 +11476,7 @@
         <v>1399</v>
       </c>
       <c r="D256" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
@@ -11520,7 +11520,7 @@
         <v>1399</v>
       </c>
       <c r="D257" s="30" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -11564,7 +11564,7 @@
         <v>1599</v>
       </c>
       <c r="D258" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
@@ -11608,7 +11608,7 @@
         <v>1599</v>
       </c>
       <c r="D259" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -11652,7 +11652,7 @@
         <v>1799</v>
       </c>
       <c r="D260" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
@@ -11696,7 +11696,7 @@
         <v>1599</v>
       </c>
       <c r="D261" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -11740,7 +11740,7 @@
         <v>1599</v>
       </c>
       <c r="D262" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E262" s="4" t="inlineStr">
         <is>
@@ -11800,7 +11800,7 @@
         <v>1499</v>
       </c>
       <c r="D264" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E264" s="4" t="inlineStr">
         <is>
@@ -11844,7 +11844,7 @@
         <v>1499</v>
       </c>
       <c r="D265" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -11888,7 +11888,7 @@
         <v>1599</v>
       </c>
       <c r="D266" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
@@ -11932,7 +11932,7 @@
         <v>1799</v>
       </c>
       <c r="D267" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -11976,7 +11976,7 @@
         <v>1499</v>
       </c>
       <c r="D268" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
@@ -12020,7 +12020,7 @@
         <v>1799</v>
       </c>
       <c r="D269" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -12064,7 +12064,7 @@
         <v>1499</v>
       </c>
       <c r="D270" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
@@ -12108,7 +12108,7 @@
         <v>1799</v>
       </c>
       <c r="D271" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -12152,7 +12152,7 @@
         <v>1599</v>
       </c>
       <c r="D272" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
@@ -12196,7 +12196,7 @@
         <v>1599</v>
       </c>
       <c r="D273" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -12240,7 +12240,7 @@
         <v>1499</v>
       </c>
       <c r="D274" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
@@ -12284,7 +12284,7 @@
         <v>1499</v>
       </c>
       <c r="D275" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -12328,7 +12328,7 @@
         <v>1499</v>
       </c>
       <c r="D276" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
@@ -12372,7 +12372,7 @@
         <v>1599</v>
       </c>
       <c r="D277" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -12432,7 +12432,7 @@
         <v>1999</v>
       </c>
       <c r="D279" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -12476,7 +12476,7 @@
         <v>1999</v>
       </c>
       <c r="D280" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E280" s="4" t="inlineStr">
         <is>
@@ -12520,7 +12520,7 @@
         <v>1999</v>
       </c>
       <c r="D281" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -12564,7 +12564,7 @@
         <v>1999</v>
       </c>
       <c r="D282" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
@@ -12608,7 +12608,7 @@
         <v>1999</v>
       </c>
       <c r="D283" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -12652,7 +12652,7 @@
         <v>1999</v>
       </c>
       <c r="D284" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E284" s="4" t="inlineStr">
         <is>
@@ -12696,7 +12696,7 @@
         <v>1999</v>
       </c>
       <c r="D285" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -12740,7 +12740,7 @@
         <v>1999</v>
       </c>
       <c r="D286" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
@@ -12784,7 +12784,7 @@
         <v>1999</v>
       </c>
       <c r="D287" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -12844,7 +12844,7 @@
         <v>1599</v>
       </c>
       <c r="D289" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -12888,7 +12888,7 @@
         <v>1799</v>
       </c>
       <c r="D290" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
@@ -12932,7 +12932,7 @@
         <v>1999</v>
       </c>
       <c r="D291" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -12976,7 +12976,7 @@
         <v>1999</v>
       </c>
       <c r="D292" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
@@ -13020,7 +13020,7 @@
         <v>1799</v>
       </c>
       <c r="D293" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -13064,7 +13064,7 @@
         <v>1999</v>
       </c>
       <c r="D294" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
@@ -13108,7 +13108,7 @@
         <v>1499</v>
       </c>
       <c r="D295" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -13152,7 +13152,7 @@
         <v>1599</v>
       </c>
       <c r="D296" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
@@ -13196,7 +13196,7 @@
         <v>1599</v>
       </c>
       <c r="D297" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -13240,7 +13240,7 @@
         <v>1999</v>
       </c>
       <c r="D298" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E298" s="4" t="inlineStr">
         <is>
@@ -13284,7 +13284,7 @@
         <v>1499</v>
       </c>
       <c r="D299" s="30" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -13328,7 +13328,7 @@
         <v>1999</v>
       </c>
       <c r="D300" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
@@ -13372,7 +13372,7 @@
         <v>1999</v>
       </c>
       <c r="D301" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -13432,7 +13432,7 @@
         <v>1599</v>
       </c>
       <c r="D303" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -13476,7 +13476,7 @@
         <v>1799</v>
       </c>
       <c r="D304" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
@@ -13520,7 +13520,7 @@
         <v>1599</v>
       </c>
       <c r="D305" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -13564,7 +13564,7 @@
         <v>1799</v>
       </c>
       <c r="D306" s="30" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="E306" s="4" t="inlineStr">
         <is>
@@ -13608,7 +13608,7 @@
         <v>1999</v>
       </c>
       <c r="D307" s="30" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -13668,7 +13668,7 @@
         <v>1599</v>
       </c>
       <c r="D309" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -13712,7 +13712,7 @@
         <v>1599</v>
       </c>
       <c r="D310" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
@@ -13756,7 +13756,7 @@
         <v>1599</v>
       </c>
       <c r="D311" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -13800,7 +13800,7 @@
         <v>1599</v>
       </c>
       <c r="D312" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
@@ -13844,7 +13844,7 @@
         <v>1599</v>
       </c>
       <c r="D313" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -13888,7 +13888,7 @@
         <v>1599</v>
       </c>
       <c r="D314" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
@@ -13932,7 +13932,7 @@
         <v>1599</v>
       </c>
       <c r="D315" s="30" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
BSD-Catalog-Master - tab 2 Reguli Preturi adaugat
</commit_message>
<xml_diff>
--- a/BSD-Catalog-Master.xlsx
+++ b/BSD-Catalog-Master.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="BSD-Catalog-Master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Reguli Preturi" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,8 +31,24 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -118,8 +135,18 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEEAF1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -127,11 +154,17 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -168,6 +201,45 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -13964,4 +14036,452 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>REGULI DE PREȚURI — Sistem BSD cu Oglinzi Dedicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>MAȘINI NOI  (yr_stop ≥ 2021 — sub 5 ani vechime)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="33" t="inlineStr">
+        <is>
+          <t>Valoare piață (EUR)</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>Pret Retail (RON)</t>
+        </is>
+      </c>
+      <c r="C4" s="33" t="inlineStr">
+        <is>
+          <t>Pret Dealer (RON)</t>
+        </is>
+      </c>
+      <c r="D4" s="33" t="inlineStr">
+        <is>
+          <t>Marjă dealer</t>
+        </is>
+      </c>
+      <c r="E4" s="33" t="inlineStr">
+        <is>
+          <t>Exemple modele</t>
+        </is>
+      </c>
+      <c r="F4" s="33" t="inlineStr">
+        <is>
+          <t>Obs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>&gt; 40.000 €</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>1.999 lei</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>1.499 lei</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="E5" s="36" t="inlineStr">
+        <is>
+          <t>MB W206, GLE V167, BMW X5/X7, Porsche</t>
+        </is>
+      </c>
+      <c r="F5" s="36" t="inlineStr">
+        <is>
+          <t>Mașini premium noi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="37" t="inlineStr">
+        <is>
+          <t>25.001–40.000 €</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>1.799 lei</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>1.349 lei</t>
+        </is>
+      </c>
+      <c r="D6" s="37" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="E6" s="38" t="inlineStr">
+        <is>
+          <t>MB W205, Audi A4/Q5, BMW X3/5, GLC</t>
+        </is>
+      </c>
+      <c r="F6" s="38" t="inlineStr">
+        <is>
+          <t>Mid-premium noi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="34" t="inlineStr">
+        <is>
+          <t>17.001–25.000 €</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>1.599 lei</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>1.199 lei</t>
+        </is>
+      </c>
+      <c r="D7" s="34" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="E7" s="36" t="inlineStr">
+        <is>
+          <t>Toyota RAV4, Honda CRV, Audi A3</t>
+        </is>
+      </c>
+      <c r="F7" s="36" t="inlineStr">
+        <is>
+          <t>Segment mediu nou</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>≤ 17.000 €</t>
+        </is>
+      </c>
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>1.399 lei</t>
+        </is>
+      </c>
+      <c r="C8" s="35" t="inlineStr">
+        <is>
+          <t>1.049 lei</t>
+        </is>
+      </c>
+      <c r="D8" s="37" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="E8" s="38" t="inlineStr">
+        <is>
+          <t>Toyota Corolla, Honda HRV, Chevrolet Trax</t>
+        </is>
+      </c>
+      <c r="F8" s="38" t="inlineStr">
+        <is>
+          <t>Segment accesibil</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="39" t="inlineStr">
+        <is>
+          <t>MAȘINI VECHI  (yr_stop &lt; 2021 — peste 5 ani vechime)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>Valoare piață (EUR)</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>Pret Retail (RON)</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>Pret Dealer (RON)</t>
+        </is>
+      </c>
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>Marjă dealer</t>
+        </is>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>Exemple modele</t>
+        </is>
+      </c>
+      <c r="F11" s="33" t="inlineStr">
+        <is>
+          <t>Obs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="40" t="inlineStr">
+        <is>
+          <t>&gt; 50.000 €</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>1.999 lei</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>1.499 lei</t>
+        </is>
+      </c>
+      <c r="D12" s="40" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="E12" s="41" t="inlineStr">
+        <is>
+          <t>Porsche, MB G-Class, Maserati vechi</t>
+        </is>
+      </c>
+      <c r="F12" s="41" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>40.001–50.000 €</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>1.799 lei</t>
+        </is>
+      </c>
+      <c r="C13" s="35" t="inlineStr">
+        <is>
+          <t>1.349 lei</t>
+        </is>
+      </c>
+      <c r="D13" s="37" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="E13" s="38" t="inlineStr">
+        <is>
+          <t>MB W222, BMW X5 vechi, Land Rover</t>
+        </is>
+      </c>
+      <c r="F13" s="38" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="40" t="inlineStr">
+        <is>
+          <t>30.001–40.000 €</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>1.599 lei</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>1.199 lei</t>
+        </is>
+      </c>
+      <c r="D14" s="40" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="E14" s="41" t="inlineStr">
+        <is>
+          <t>MB W212 facelift, Audi A6 vechi, Lexus RX</t>
+        </is>
+      </c>
+      <c r="F14" s="41" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>20.001–30.000 €</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>1.499 lei</t>
+        </is>
+      </c>
+      <c r="C15" s="35" t="inlineStr">
+        <is>
+          <t>1.099 lei</t>
+        </is>
+      </c>
+      <c r="D15" s="37" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="E15" s="38" t="inlineStr">
+        <is>
+          <t>Toyota Highlander, Honda Pilot, Ford Edge</t>
+        </is>
+      </c>
+      <c r="F15" s="38" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="40" t="inlineStr">
+        <is>
+          <t>10.001–20.000 €</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>1.399 lei</t>
+        </is>
+      </c>
+      <c r="C16" s="35" t="inlineStr">
+        <is>
+          <t>1.049 lei</t>
+        </is>
+      </c>
+      <c r="D16" s="40" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="E16" s="41" t="inlineStr">
+        <is>
+          <t>Toyota Camry vechi, Nissan Patrol, MB W204</t>
+        </is>
+      </c>
+      <c r="F16" s="41" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t>≤ 10.000 €</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>1.199 lei</t>
+        </is>
+      </c>
+      <c r="C17" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  899 lei</t>
+        </is>
+      </c>
+      <c r="D17" s="37" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="E17" s="38" t="inlineStr">
+        <is>
+          <t>Toyota Verso, Nissan Tiida, Chery vechi</t>
+        </is>
+      </c>
+      <c r="F17" s="38" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="42" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="43" t="inlineStr">
+        <is>
+          <t>• Prețul dealer = prețul retail - 25%, rotunjit la cel mai apropiat multiplu de 50 lei</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="43" t="inlineStr">
+        <is>
+          <t>• Valoarea de piață = valoarea medie estimată pentru modelul respectiv (uzat/semi-nou), EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="43" t="inlineStr">
+        <is>
+          <t>• Criteriul 'nou/vechi' = dacă yr_stop (ultimul an de fabricație al generației) ≥ 2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="43" t="inlineStr">
+        <is>
+          <t>• Valorile de piață sunt estimate și pot fi ajustate manual în tab-ul principal</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A20:F20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
BSD-Catalog-Master - titluri SEO actualizate (senzor unghi mort + oglinda dedicata)
</commit_message>
<xml_diff>
--- a/BSD-Catalog-Master.xlsx
+++ b/BSD-Catalog-Master.xlsx
@@ -697,7 +697,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz C-Class W204 2007-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz C-Class W204 2007-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C3" s="29" t="n">
@@ -741,7 +741,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz E-Class W212 2009-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz E-Class W212 2009-2016 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C4" s="29" t="n">
@@ -785,7 +785,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz GLK X204 2008-2015 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz GLK X204 2008-2015 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C5" s="29" t="n">
@@ -829,7 +829,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz GLA X156 2013-2020 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz GLA X156 2013-2020 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C6" s="29" t="n">
@@ -873,7 +873,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz A-Class W176 2012-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz A-Class W176 2012-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C7" s="29" t="n">
@@ -917,7 +917,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz B-Class W246 2011-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz B-Class W246 2011-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C8" s="29" t="n">
@@ -961,7 +961,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz CLA C117 2013-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz CLA C117 2013-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C9" s="29" t="n">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz S-Class W221 2005-2013 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz S-Class W221 2005-2013 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C10" s="29" t="n">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz CLS C218 2011-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz CLS C218 2011-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C11" s="29" t="n">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz ML W164 2005-2011 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz ML W164 2005-2011 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C12" s="29" t="n">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz GLE W166 2015-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz GLE W166 2015-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C13" s="29" t="n">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz GLS X166 2015-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz GLS X166 2015-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C14" s="29" t="n">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz GL X166 2012-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz GL X166 2012-2016 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C15" s="29" t="n">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz R-Class W251 2005-2017 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz R-Class W251 2005-2017 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C16" s="29" t="n">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz G-Class W463 2008-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz G-Class W463 2008-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C17" s="29" t="n">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz C-Class W205 2014-2021 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz C-Class W205 2014-2021 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C18" s="29" t="n">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz E-Class W213 2016-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz E-Class W213 2016-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C19" s="29" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz GLA H247 2020-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz GLA H247 2020-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C20" s="29" t="n">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz GLC X253 2015-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz GLC X253 2015-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C21" s="29" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz GLB X247 2019-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz GLB X247 2019-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C22" s="29" t="n">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz B-Class W247 2018-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz B-Class W247 2018-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C23" s="29" t="n">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz EQC N293 2019-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz EQC N293 2019-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C24" s="29" t="n">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz EQA H243 2021-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz EQA H243 2021-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C25" s="29" t="n">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz EQB X243 2021-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz EQB X243 2021-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C26" s="29" t="n">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz S-Class W222 2013-2020 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz S-Class W222 2013-2020 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C27" s="29" t="n">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz CLS C257 2018-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz CLS C257 2018-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C28" s="29" t="n">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz GT AMG C190 2014-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz GT AMG C190 2014-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C29" s="29" t="n">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz A-Class W177 2018-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz A-Class W177 2018-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C30" s="29" t="n">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz CLA C118 2019-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz CLA C118 2019-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C31" s="29" t="n">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz Vito W447 2014-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz Vito W447 2014-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C32" s="29" t="n">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz V-Class W447 2014-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz V-Class W447 2014-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C33" s="29" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz EQV W447 2020-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz EQV W447 2020-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C34" s="29" t="n">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz G-Class W463 2012-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz G-Class W463 2012-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C35" s="29" t="n">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz C-Class W206 2021-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz C-Class W206 2021-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C36" s="29" t="n">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz GLC X254 2022-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz GLC X254 2022-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C37" s="29" t="n">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz EQS V297 2021-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz EQS V297 2021-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C38" s="29" t="n">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz E-Class W214 2023-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz E-Class W214 2023-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C39" s="29" t="n">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz S-Class W223 2020-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz S-Class W223 2020-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C40" s="29" t="n">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz S Maybach W223 2020-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz S Maybach W223 2020-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C41" s="29" t="n">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz CLE W236 2023-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz CLE W236 2023-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C42" s="29" t="n">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz GLE V167 2018-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz GLE V167 2018-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C43" s="29" t="n">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz GLS X167 2019-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz GLS X167 2019-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C44" s="29" t="n">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes-Benz G-Class W463 2018-2026 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mercedes-Benz G-Class W463 2018-2026 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C45" s="29" t="n">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A6L 2012-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A6L 2012-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C47" s="29" t="n">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi S6 2013-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi S6 2013-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C48" s="29" t="n">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A6 2013-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A6 2013-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C49" s="29" t="n">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A4L 2017-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A4L 2017-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C50" s="29" t="n">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A5 2017-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A5 2017-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C51" s="29" t="n">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi RS4 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi RS4 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C52" s="29" t="n">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Unghi mort Audi RS5 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi RS5 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C53" s="29" t="n">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A4 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A4 2016-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C54" s="29" t="n">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Unghi mort Audi S4 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi S4 2016-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C55" s="29" t="n">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi S5 2017-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi S5 2017-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C56" s="29" t="n">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A3 2014-2020 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A3 2014-2020 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C57" s="29" t="n">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi S3 2015-2020 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi S3 2015-2020 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C58" s="29" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A6L 2009-2011 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A6L 2009-2011 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C59" s="29" t="n">
@@ -3177,7 +3177,7 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi Q3 2012-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi Q3 2012-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C60" s="29" t="n">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A8 2008-2009 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A8 2008-2009 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C61" s="29" t="n">
@@ -3265,7 +3265,7 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A4L 2009-2012 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A4L 2009-2012 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C62" s="29" t="n">
@@ -3309,7 +3309,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A4 2013-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A4 2013-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C63" s="29" t="n">
@@ -3353,7 +3353,7 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A4L 2013-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A4L 2013-2016 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C64" s="29" t="n">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A5 2012-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A5 2012-2016 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C65" s="29" t="n">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi S5 2010-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi S5 2010-2016 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C66" s="29" t="n">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A3 2013-2013 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A3 2013-2013 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C67" s="29" t="n">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi RS5 2011-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi RS5 2011-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C68" s="29" t="n">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Unghi mort Audi Q5 2010-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi Q5 2010-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C69" s="29" t="n">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi SQ5 2010-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi SQ5 2010-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C70" s="29" t="n">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Unghi mort Audi Q7 2006-2015 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi Q7 2006-2015 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C71" s="29" t="n">
@@ -3705,7 +3705,7 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi Q7 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi Q7 2016-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C72" s="29" t="n">
@@ -3749,7 +3749,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Unghi mort Audi Q5L 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi Q5L 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C73" s="29" t="n">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi Q2L 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi Q2L 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C74" s="29" t="n">
@@ -3837,7 +3837,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Unghi mort Audi Q3 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi Q3 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C75" s="29" t="n">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A6L 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A6L 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C76" s="29" t="n">
@@ -3925,7 +3925,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A7 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A7 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C77" s="29" t="n">
@@ -3969,7 +3969,7 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A8L 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A8L 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C78" s="29" t="n">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A6 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A6 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C79" s="29" t="n">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi RS7 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi RS7 2021-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C80" s="29" t="n">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Unghi mort Audi S8 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi S8 2021-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C81" s="29" t="n">
@@ -4145,7 +4145,7 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A1 2012-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A1 2012-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C82" s="29" t="n">
@@ -4189,7 +4189,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A1 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A1 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C83" s="29" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A3 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A3 2021-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C84" s="29" t="n">
@@ -4277,7 +4277,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Unghi mort Audi e-tron 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi e-tron 2021-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C85" s="29" t="n">
@@ -4321,7 +4321,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi A8 2011-2017 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi A8 2011-2017 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C86" s="29" t="n">
@@ -4365,7 +4365,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Unghi mort Audi S8 2013-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi S8 2013-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C87" s="29" t="n">
@@ -4409,7 +4409,7 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi Q6 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi Q6 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C88" s="29" t="n">
@@ -4453,7 +4453,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Unghi mort Audi Q8 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi Q8 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C89" s="29" t="n">
@@ -4497,7 +4497,7 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Audi Q4 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi Q4 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C90" s="29" t="n">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Unghi mort Audi Q5 e-tron 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Audi Q5 e-tron 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C91" s="29" t="n">
@@ -4601,7 +4601,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 5 2011-2017 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 5 2011-2017 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C93" s="29" t="n">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 7 2009-2015 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 7 2009-2015 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C94" s="29" t="n">
@@ -4689,7 +4689,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 5 GT 2010-2017 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 5 GT 2010-2017 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C95" s="29" t="n">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 6 2012-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 6 2012-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C96" s="29" t="n">
@@ -4777,7 +4777,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 3 2013-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 3 2013-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C97" s="29" t="n">
@@ -4821,7 +4821,7 @@
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW X1 2013-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW X1 2013-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C98" s="29" t="n">
@@ -4865,7 +4865,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 4 2013-2020 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 4 2013-2020 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C99" s="29" t="n">
@@ -4909,7 +4909,7 @@
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 3 GT 2013-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 3 GT 2013-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C100" s="29" t="n">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 2 2014-2021 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 2 2014-2021 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C101" s="29" t="n">
@@ -4997,7 +4997,7 @@
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 2 2018-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 2 2018-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C102" s="29" t="n">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 1 2017-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 1 2017-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C103" s="29" t="n">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW X2 2018-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW X2 2018-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C104" s="29" t="n">
@@ -5129,7 +5129,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Unghi mort BMW Z4 2019-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW Z4 2019-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C105" s="29" t="n">
@@ -5173,7 +5173,7 @@
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW 2019 I3  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW 2019 I3  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C106" s="29" t="n">
@@ -5213,7 +5213,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Unghi mort BMW X3 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW X3 2014-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C107" s="29" t="n">
@@ -5257,7 +5257,7 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW X4 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW X4 2014-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C108" s="29" t="n">
@@ -5301,7 +5301,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Unghi mort BMW X5 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW X5 2014-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C109" s="29" t="n">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW X6 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW X6 2015-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C110" s="29" t="n">
@@ -5389,7 +5389,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Unghi mort BMW X7 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW X7 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C111" s="29" t="n">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW IX3 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW IX3 2020-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C112" s="29" t="n">
@@ -5477,7 +5477,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Unghi mort BMW X4M 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW X4M 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C113" s="29" t="n">
@@ -5521,7 +5521,7 @@
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW X3M 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW X3M 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C114" s="29" t="n">
@@ -5565,7 +5565,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Unghi mort BMW X5M 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW X5M 2015-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C115" s="29" t="n">
@@ -5609,7 +5609,7 @@
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW X6M 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW X6M 2015-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C116" s="29" t="n">
@@ -5653,7 +5653,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 7 2016-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 7 2016-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C117" s="29" t="n">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 5 2018-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 5 2018-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C118" s="29" t="n">
@@ -5741,7 +5741,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 4 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 4 2021-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C119" s="29" t="n">
@@ -5785,7 +5785,7 @@
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 6 GT 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 6 GT 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C120" s="29" t="n">
@@ -5829,7 +5829,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 3 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 3 2020-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C121" s="29" t="n">
@@ -5873,7 +5873,7 @@
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 8 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 8 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C122" s="29" t="n">
@@ -5917,7 +5917,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW 2 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW 2 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C123" s="29" t="n">
@@ -5961,7 +5961,7 @@
       </c>
       <c r="B124" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW M4 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW M4 2021-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C124" s="29" t="n">
@@ -6005,7 +6005,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW I3 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW I3 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C125" s="29" t="n">
@@ -6049,7 +6049,7 @@
       </c>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW I4 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW I4 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C126" s="29" t="n">
@@ -6093,7 +6093,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW M3 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW M3 2021-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C127" s="29" t="n">
@@ -6137,7 +6137,7 @@
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW 2019  BMW M8  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW 2019  BMW M8  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C128" s="29" t="n">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Unghi mort BMW BMW M5 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW BMW M5 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C129" s="29" t="n">
@@ -6221,7 +6221,7 @@
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW MINI 2015-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW MINI 2015-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C130" s="29" t="n">
@@ -6265,7 +6265,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Unghi mort BMW MINI CLUBMAN 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW MINI CLUBMAN 2016-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C131" s="29" t="n">
@@ -6309,7 +6309,7 @@
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW MINI COUNTRYMAN 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW MINI COUNTRYMAN 2015-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C132" s="29" t="n">
@@ -6353,7 +6353,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Unghi mort BMW 2023 BMW 7  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW 2023 BMW 7  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C133" s="29" t="n">
@@ -6391,7 +6391,7 @@
       </c>
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW 2024 BMW 5  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW 2024 BMW 5  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C134" s="29" t="n">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Unghi mort BMW 2023 BMW I7  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW 2023 BMW I7  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C135" s="29" t="n">
@@ -6469,7 +6469,7 @@
       </c>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW X5 2008-2013 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW X5 2008-2013 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C136" s="29" t="n">
@@ -6513,7 +6513,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Unghi mort BMW X6 2009-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW X6 2009-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C137" s="29" t="n">
@@ -6557,7 +6557,7 @@
       </c>
       <c r="B138" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW 2O1O-2014 X5M  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW 2O1O-2014 X5M  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C138" s="29" t="n">
@@ -6597,7 +6597,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Unghi mort BMW X6M 2013-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW X6M 2013-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C139" s="29" t="n">
@@ -6641,7 +6641,7 @@
       </c>
       <c r="B140" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort BMW 2013 C5  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort BMW 2013 C5  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C140" s="29" t="n">
@@ -6697,7 +6697,7 @@
       </c>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Wildlander 2020-2025 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Wildlander 2020-2025 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C142" s="29" t="n">
@@ -6741,7 +6741,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Frontlander 2022-2025 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Frontlander 2022-2025 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C143" s="29" t="n">
@@ -6785,7 +6785,7 @@
       </c>
       <c r="B144" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Venza 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Venza 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C144" s="29" t="n">
@@ -6829,7 +6829,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Rav4 2020-2025 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Rav4 2020-2025 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C145" s="29" t="n">
@@ -6873,7 +6873,7 @@
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Toyota cross 2022-2025 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Toyota cross 2022-2025 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C146" s="29" t="n">
@@ -6917,7 +6917,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Toyota Hilux 2021-2025 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Toyota Hilux 2021-2025 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C147" s="29" t="n">
@@ -6961,7 +6961,7 @@
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota CROWN KLUGER 2021-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota CROWN KLUGER 2021-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C148" s="29" t="n">
@@ -7005,7 +7005,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Highlander 2015-2021 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Highlander 2015-2021 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C149" s="29" t="n">
@@ -7049,7 +7049,7 @@
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Toyota Alphard 30 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Toyota Alphard 30 2015-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C150" s="29" t="n">
@@ -7093,7 +7093,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Toyota Vellfire 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Toyota Vellfire 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C151" s="29" t="n">
@@ -7137,7 +7137,7 @@
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota 4 Runner 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota 4 Runner 2015-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C152" s="29" t="n">
@@ -7181,7 +7181,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Fortuner 2015-2025 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Fortuner 2015-2025 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C153" s="29" t="n">
@@ -7225,7 +7225,7 @@
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Tacoma 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Tacoma 2020-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C154" s="29" t="n">
@@ -7269,7 +7269,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Highlander 2022-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Highlander 2022-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C155" s="29" t="n">
@@ -7313,7 +7313,7 @@
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Sienna 2021-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Sienna 2021-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C156" s="29" t="n">
@@ -7357,7 +7357,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Verso 2009-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Verso 2009-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C157" s="29" t="n">
@@ -7401,7 +7401,7 @@
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Rav4 2009-2012 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Rav4 2009-2012 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C158" s="29" t="n">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Corolla 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Corolla 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C159" s="29" t="n">
@@ -7489,7 +7489,7 @@
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Prado 2010-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Prado 2010-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C160" s="29" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Land Cruiser LC200 2010-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Land Cruiser LC200 2010-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C161" s="29" t="n">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Land Cruiser LC300 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Land Cruiser LC300 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C162" s="29" t="n">
@@ -7621,7 +7621,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Land Cruiser LC100 2007-2009 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Land Cruiser LC100 2007-2009 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C163" s="29" t="n">
@@ -7665,7 +7665,7 @@
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Rav4 2013-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Rav4 2013-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C164" s="29" t="n">
@@ -7709,7 +7709,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Corolla 2014-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Corolla 2014-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C165" s="29" t="n">
@@ -7753,7 +7753,7 @@
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Camry 2009-2011 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Camry 2009-2011 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C166" s="29" t="n">
@@ -7797,7 +7797,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Yaris 2009-2011 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Yaris 2009-2011 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C167" s="29" t="n">
@@ -7841,7 +7841,7 @@
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Corolla 2008-2013 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Corolla 2008-2013 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C168" s="29" t="n">
@@ -7885,7 +7885,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota 2010 Prius  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota 2010 Prius  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C169" s="29" t="n">
@@ -7923,7 +7923,7 @@
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Toyota Hilux 2005-2015 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Toyota Hilux 2005-2015 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C170" s="29" t="n">
@@ -7983,7 +7983,7 @@
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus ES 2013-2017 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus ES 2013-2017 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C172" s="29" t="n">
@@ -8027,7 +8027,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus CT 2011-2017 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus CT 2011-2017 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C173" s="29" t="n">
@@ -8071,7 +8071,7 @@
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus IS 2013-2017 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus IS 2013-2017 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C174" s="29" t="n">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus GS 2012-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus GS 2012-2016 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C175" s="29" t="n">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus LS 2013-2017 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus LS 2013-2017 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C176" s="29" t="n">
@@ -8203,7 +8203,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus NX 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus NX 2014-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C177" s="29" t="n">
@@ -8247,7 +8247,7 @@
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus RX 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus RX 2016-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C178" s="29" t="n">
@@ -8291,7 +8291,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus LM 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus LM 2020-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C179" s="29" t="n">
@@ -8335,7 +8335,7 @@
       </c>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus RZ 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus RZ 2023-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C180" s="29" t="n">
@@ -8379,7 +8379,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus RX 2009-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus RX 2009-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C181" s="29" t="n">
@@ -8423,7 +8423,7 @@
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus LS 2009-2012 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus LS 2009-2012 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C182" s="29" t="n">
@@ -8467,7 +8467,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus ES 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus ES 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C183" s="29" t="n">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus UX 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus UX 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C184" s="29" t="n">
@@ -8555,7 +8555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus LC 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus LC 2016-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C185" s="29" t="n">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus LS 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus LS 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C186" s="29" t="n">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus GX 2010-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus GX 2010-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C187" s="29" t="n">
@@ -8687,7 +8687,7 @@
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus ES 2006-2012 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus ES 2006-2012 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C188" s="29" t="n">
@@ -8731,7 +8731,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Unghi mort Lexus RX 2006-2008 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Lexus RX 2006-2008 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C189" s="29" t="n">
@@ -8791,7 +8791,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Unghi mort Honda HRV 2015-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda HRV 2015-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C191" s="29" t="n">
@@ -8835,7 +8835,7 @@
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda X-RV 2015-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda X-RV 2015-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C192" s="29" t="n">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Breeze 2020-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Breeze 2020-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C193" s="29" t="n">
@@ -8923,7 +8923,7 @@
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda CRV G5 2017-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda CRV G5 2017-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C194" s="29" t="n">
@@ -8967,7 +8967,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Unghi mort Honda CRV hybrid 2021-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda CRV hybrid 2021-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C195" s="29" t="n">
@@ -9011,7 +9011,7 @@
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Crosstour 2010-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Crosstour 2010-2016 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C196" s="29" t="n">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Honda Fit 2014-2020 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Honda Fit 2014-2020 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C197" s="29" t="n">
@@ -9099,7 +9099,7 @@
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Honda Jazz 2015-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Honda Jazz 2015-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C198" s="29" t="n">
@@ -9143,7 +9143,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Unghi mort Honda City 2015-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda City 2015-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C199" s="29" t="n">
@@ -9187,7 +9187,7 @@
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Honda Fit 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Honda Fit 2021-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C200" s="29" t="n">
@@ -9231,7 +9231,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Honda Jazz 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Honda Jazz 2020-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C201" s="29" t="n">
@@ -9275,7 +9275,7 @@
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda WRV 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda WRV 2023-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C202" s="29" t="n">
@@ -9319,7 +9319,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Unghi mort Honda 2023 BRV  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda 2023 BRV  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C203" s="29" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Honda Fit 2008-2013 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Honda Fit 2008-2013 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C204" s="29" t="n">
@@ -9401,7 +9401,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Unghi mort Honda City 2009-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda City 2009-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C205" s="29" t="n">
@@ -9445,7 +9445,7 @@
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Honda Civic 10th 2016-2021 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Honda Civic 10th 2016-2021 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C206" s="29" t="n">
@@ -9489,7 +9489,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Unghi mort Honda ODYSSEY 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda ODYSSEY 2015-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C207" s="29" t="n">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda ODYSSEY 2011-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda ODYSSEY 2011-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C208" s="29" t="n">
@@ -9577,7 +9577,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Accord 10th ( without right camera) 2018-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Accord 10th ( without right camera) 2018-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C209" s="29" t="n">
@@ -9621,7 +9621,7 @@
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda 2024  Accord 11th (without right camera)  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda 2024  Accord 11th (without right camera)  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C210" s="29" t="n">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Inspire 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Inspire 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C211" s="29" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Accord 10th ( with right camera) 2018-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Accord 10th ( with right camera) 2018-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C212" s="29" t="n">
@@ -9749,7 +9749,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Unghi mort Honda 2024  Accord 11th (with right camera)  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda 2024  Accord 11th (with right camera)  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C213" s="29" t="n">
@@ -9787,7 +9787,7 @@
       </c>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Inspire 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Inspire 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C214" s="29" t="n">
@@ -9831,7 +9831,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Unghi mort Honda Honda Civic 11th 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda Honda Civic 11th 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C215" s="29" t="n">
@@ -9875,7 +9875,7 @@
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda HRV 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda HRV 2023-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C216" s="29" t="n">
@@ -9919,7 +9919,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Unghi mort Honda ZRV 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda ZRV 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C217" s="29" t="n">
@@ -9963,7 +9963,7 @@
       </c>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda e:NP1 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda e:NP1 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C218" s="29" t="n">
@@ -10007,7 +10007,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Unghi mort Honda CRV 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda CRV 2023-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C219" s="29" t="n">
@@ -10051,7 +10051,7 @@
       </c>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Honda XRV 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda XRV 2023-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C220" s="29" t="n">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Unghi mort Honda e:NS1 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Honda e:NS1 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C221" s="29" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Unghi mort Ford Mondeo 2013-2021 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Ford Mondeo 2013-2021 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C223" s="29" t="n">
@@ -10199,7 +10199,7 @@
       </c>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Ford Mondeo 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Ford Mondeo 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C224" s="29" t="n">
@@ -10243,7 +10243,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Unghi mort Ford Mondeo 2008-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Ford Mondeo 2008-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C225" s="29" t="n">
@@ -10287,7 +10287,7 @@
       </c>
       <c r="B226" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Ford Edge 2015-2020 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Ford Edge 2015-2020 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C226" s="29" t="n">
@@ -10331,7 +10331,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Unghi mort Ford Edge PLUS 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Ford Edge PLUS 2021-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C227" s="29" t="n">
@@ -10375,7 +10375,7 @@
       </c>
       <c r="B228" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Ford Kuga 2013-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Ford Kuga 2013-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C228" s="29" t="n">
@@ -10419,7 +10419,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Unghi mort Ford EcoSport 2013-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Ford EcoSport 2013-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C229" s="29" t="n">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Ford Escape 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Ford Escape 2020-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C230" s="29" t="n">
@@ -10507,7 +10507,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Unghi mort Ford Escort 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Ford Escort 2021-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C231" s="29" t="n">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Ford Explorer 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Ford Explorer 2020-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C232" s="29" t="n">
@@ -10595,7 +10595,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Unghi mort Ford Everest 2016-2020 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Ford Everest 2016-2020 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C233" s="29" t="n">
@@ -10655,7 +10655,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Equinox 2017-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Equinox 2017-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C235" s="29" t="n">
@@ -10699,7 +10699,7 @@
       </c>
       <c r="B236" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Malibu 2012-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Malibu 2012-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C236" s="29" t="n">
@@ -10743,7 +10743,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Malibu XL 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Malibu XL 2016-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C237" s="29" t="n">
@@ -10787,7 +10787,7 @@
       </c>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet TRAX 2014-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet TRAX 2014-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C238" s="29" t="n">
@@ -10831,7 +10831,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet TRAX 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet TRAX 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C239" s="29" t="n">
@@ -10875,7 +10875,7 @@
       </c>
       <c r="B240" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Cruze 2009-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Cruze 2009-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C240" s="29" t="n">
@@ -10919,7 +10919,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Cruze 2015-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Cruze 2015-2016 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C241" s="29" t="n">
@@ -10963,7 +10963,7 @@
       </c>
       <c r="B242" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Cruze 2017-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Cruze 2017-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C242" s="29" t="n">
@@ -11007,7 +11007,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Cruze 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Cruze 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C243" s="29" t="n">
@@ -11051,7 +11051,7 @@
       </c>
       <c r="B244" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Cruze 2016-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Cruze 2016-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C244" s="29" t="n">
@@ -11095,7 +11095,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Blazer 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Blazer 2020-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C245" s="29" t="n">
@@ -11139,7 +11139,7 @@
       </c>
       <c r="B246" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Orlando 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Orlando 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C246" s="29" t="n">
@@ -11183,7 +11183,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Lova RV 2016-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Lova RV 2016-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C247" s="29" t="n">
@@ -11227,7 +11227,7 @@
       </c>
       <c r="B248" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Sail 3 2015-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Sail 3 2015-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C248" s="29" t="n">
@@ -11271,7 +11271,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet AVEO 2011-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet AVEO 2011-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C249" s="29" t="n">
@@ -11315,7 +11315,7 @@
       </c>
       <c r="B250" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Trailblazer 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Trailblazer 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C250" s="29" t="n">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet 2019 Corolado  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet 2019 Corolado  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C251" s="29" t="n">
@@ -11397,7 +11397,7 @@
       </c>
       <c r="B252" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Chevrolet Menlo 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chevrolet Menlo 2020-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C252" s="29" t="n">
@@ -11457,7 +11457,7 @@
       </c>
       <c r="B254" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Nissan 20212-2025 Patrol Y63 Y62  - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Nissan 20212-2025 Patrol Y63 Y62  — oglindă dedicată</t>
         </is>
       </c>
       <c r="C254" s="29" t="n">
@@ -11497,7 +11497,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Unghi mort Nissan Nissan Sylphy 2012-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Nissan Nissan Sylphy 2012-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C255" s="29" t="n">
@@ -11541,7 +11541,7 @@
       </c>
       <c r="B256" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Nissan Nissan Altima 2013-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Nissan Nissan Altima 2013-2018 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C256" s="29" t="n">
@@ -11585,7 +11585,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Unghi mort Nissan Nissan TIIDA 2016-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Nissan Nissan TIIDA 2016-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C257" s="29" t="n">
@@ -11629,7 +11629,7 @@
       </c>
       <c r="B258" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Nissan Altima 2019-2025 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Nissan Altima 2019-2025 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C258" s="29" t="n">
@@ -11673,7 +11673,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Unghi mort Nissan Qashqai 2016-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Nissan Qashqai 2016-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C259" s="29" t="n">
@@ -11717,7 +11717,7 @@
       </c>
       <c r="B260" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Nissan Murano 2015-2025 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Nissan Murano 2015-2025 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C260" s="29" t="n">
@@ -11761,7 +11761,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Unghi mort Nissan Nissan X-Trail 2022-2025 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Nissan Nissan X-Trail 2022-2025 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C261" s="29" t="n">
@@ -11805,7 +11805,7 @@
       </c>
       <c r="B262" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Nissan Nissan X-Trail 2014-2021 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Nissan Nissan X-Trail 2014-2021 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C262" s="29" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B264" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda Mazda 3 2014-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda Mazda 3 2014-2016 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C264" s="29" t="n">
@@ -11909,7 +11909,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda Mazda 3 2017-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda Mazda 3 2017-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C265" s="29" t="n">
@@ -11953,7 +11953,7 @@
       </c>
       <c r="B266" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda Mazda 6 2014-2021 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda Mazda 6 2014-2021 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C266" s="29" t="n">
@@ -11997,7 +11997,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda CX4 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda CX4 2016-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C267" s="29" t="n">
@@ -12041,7 +12041,7 @@
       </c>
       <c r="B268" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda CX5 2015-2017 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda CX5 2015-2017 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C268" s="29" t="n">
@@ -12085,7 +12085,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda CX5 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda CX5 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C269" s="29" t="n">
@@ -12129,7 +12129,7 @@
       </c>
       <c r="B270" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda CX3 2016-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda CX3 2016-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C270" s="29" t="n">
@@ -12173,7 +12173,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda CX8 2018-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda CX8 2018-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C271" s="29" t="n">
@@ -12217,7 +12217,7 @@
       </c>
       <c r="B272" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda Mazda 3 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda Mazda 3 2020-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C272" s="29" t="n">
@@ -12261,7 +12261,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda Mazda Axela 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda Mazda Axela 2020-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C273" s="29" t="n">
@@ -12305,7 +12305,7 @@
       </c>
       <c r="B274" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda Mazda 2 2007-2012 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda Mazda 2 2007-2012 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C274" s="29" t="n">
@@ -12349,7 +12349,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda Mazda 3 2011-2013 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda Mazda 3 2011-2013 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C275" s="29" t="n">
@@ -12393,7 +12393,7 @@
       </c>
       <c r="B276" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda Mazda 6 2009-2015 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda Mazda 6 2009-2015 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C276" s="29" t="n">
@@ -12437,7 +12437,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Unghi mort Mazda Mazda CX30 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Mazda Mazda CX30 2020-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C277" s="29" t="n">
@@ -12497,7 +12497,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Unghi mort Porsche Panamera 2009-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Porsche Panamera 2009-2016 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C279" s="29" t="n">
@@ -12541,7 +12541,7 @@
       </c>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Porsche Cayenne 2011-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Porsche Cayenne 2011-2014 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C280" s="29" t="n">
@@ -12585,7 +12585,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Unghi mort Porsche Cayenne 2015-2017 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Porsche Cayenne 2015-2017 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C281" s="29" t="n">
@@ -12629,7 +12629,7 @@
       </c>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Porsche Panamera 2017-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Porsche Panamera 2017-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C282" s="29" t="n">
@@ -12673,7 +12673,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Unghi mort Porsche Cayenne 2018-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Porsche Cayenne 2018-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C283" s="29" t="n">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Porsche 718/Boxster 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Porsche 718/Boxster 2016-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C284" s="29" t="n">
@@ -12761,7 +12761,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Unghi mort Porsche Macan 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Porsche Macan 2014-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C285" s="29" t="n">
@@ -12805,7 +12805,7 @@
       </c>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Porsche Taycan 2019-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Porsche Taycan 2019-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C286" s="29" t="n">
@@ -12849,7 +12849,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Unghi mort Porsche 911 2020-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Porsche 911 2020-2023 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C287" s="29" t="n">
@@ -12909,7 +12909,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Freelander 2015-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Freelander 2015-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C289" s="29" t="n">
@@ -12953,7 +12953,7 @@
       </c>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Range Rover Evoque 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Range Rover Evoque 2014-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C290" s="29" t="n">
@@ -12997,7 +12997,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Range Rover 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Range Rover 2014-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C291" s="29" t="n">
@@ -13041,7 +13041,7 @@
       </c>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Range Rover sport 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Range Rover sport 2014-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C292" s="29" t="n">
@@ -13085,7 +13085,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Discover 4 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Discover 4 2014-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C293" s="29" t="n">
@@ -13129,7 +13129,7 @@
       </c>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Discover 5 2014-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Discover 5 2014-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C294" s="29" t="n">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Freelander 2 2010-2015 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Freelander 2 2010-2015 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C295" s="29" t="n">
@@ -13217,7 +13217,7 @@
       </c>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Discover 4 2010-2013 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Discover 4 2010-2013 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C296" s="29" t="n">
@@ -13261,7 +13261,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Range Rover Evoque 2011-2013 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Range Rover Evoque 2011-2013 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C297" s="29" t="n">
@@ -13305,7 +13305,7 @@
       </c>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Discover 3 2005-2009 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Discover 3 2005-2009 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C298" s="29" t="n">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Freelander 2 2007-2009 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Freelander 2 2007-2009 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C299" s="29" t="n">
@@ -13393,7 +13393,7 @@
       </c>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Range Rover 2005-2008 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Range Rover 2005-2008 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C300" s="29" t="n">
@@ -13437,7 +13437,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Unghi mort Land Rover Range Rover sport 2005-2009 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Land Rover Range Rover sport 2005-2009 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C301" s="29" t="n">
@@ -13497,7 +13497,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Unghi mort Maserati Ghibli 2014-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Maserati Ghibli 2014-2016 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C303" s="29" t="n">
@@ -13541,7 +13541,7 @@
       </c>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Maserati Quattroporte 2014-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Maserati Quattroporte 2014-2016 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C304" s="29" t="n">
@@ -13585,7 +13585,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Unghi mort Maserati Ghibli 2017-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Maserati Ghibli 2017-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C305" s="29" t="n">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Maserati Quattroporte 2017-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Maserati Quattroporte 2017-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C306" s="29" t="n">
@@ -13673,7 +13673,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Unghi mort Maserati Levante 2016-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Maserati Levante 2016-2019 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C307" s="29" t="n">
@@ -13733,7 +13733,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Unghi mort Chery Tiggo 8 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chery Tiggo 8 2021-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C309" s="29" t="n">
@@ -13777,7 +13777,7 @@
       </c>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Chery Tiggo 8 PLUS 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chery Tiggo 8 PLUS 2021-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C310" s="29" t="n">
@@ -13821,7 +13821,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Unghi mort Chery Tiggo 7 2020-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chery Tiggo 7 2020-2022 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C311" s="29" t="n">
@@ -13865,7 +13865,7 @@
       </c>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Chery Tiggo E 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chery Tiggo E 2019-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C312" s="29" t="n">
@@ -13909,7 +13909,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Unghi mort Chery Tiggo 8 pro 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chery Tiggo 8 pro 2022-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C313" s="29" t="n">
@@ -13953,7 +13953,7 @@
       </c>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>Unghi mort Chery Tiggo 7 plus 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chery Tiggo 7 plus 2023-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C314" s="29" t="n">
@@ -13997,7 +13997,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Unghi mort Chery Tiggo 9 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Senzor unghi mort Chery Tiggo 9 2023-2024 — oglindă dedicată</t>
         </is>
       </c>
       <c r="C315" s="29" t="n">

</xml_diff>

<commit_message>
BSD Catalog Master - adaugat 70 produse Volkswagen (total 385)
</commit_message>
<xml_diff>
--- a/BSD-Catalog-Master.xlsx
+++ b/BSD-Catalog-Master.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,8 +47,13 @@
       <i val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001B5E20"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -145,6 +150,11 @@
         <fgColor rgb="00DEEAF1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -164,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -241,6 +251,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -606,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J315"/>
+  <dimension ref="A1:J387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14031,6 +14042,3093 @@
       </c>
       <c r="J315" t="n">
         <v>2024</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="44" t="inlineStr">
+        <is>
+          <t>▶  VOLKSWAGEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-01-V1</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen TACQUA 2020-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C318" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D318" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>BSD-VW-01</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>TACQUA</t>
+        </is>
+      </c>
+      <c r="I318" t="n">
+        <v>2020</v>
+      </c>
+      <c r="J318" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-01-V2</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen TAYRON 2020-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D319" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>BSD-VW-01</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>TAYRON</t>
+        </is>
+      </c>
+      <c r="I319" t="n">
+        <v>2020</v>
+      </c>
+      <c r="J319" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-01-V3</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen TAYRON X 2020-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D320" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>BSD-VW-01</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>TAYRON X</t>
+        </is>
+      </c>
+      <c r="I320" t="n">
+        <v>2020</v>
+      </c>
+      <c r="J320" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-01-V4</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen TALAGON 2021-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D321" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>BSD-VW-01</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>TALAGON</t>
+        </is>
+      </c>
+      <c r="I321" t="n">
+        <v>2021</v>
+      </c>
+      <c r="J321" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-01-V5</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Tiguan L 2019-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D322" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>BSD-VW-01</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>Tiguan L</t>
+        </is>
+      </c>
+      <c r="I322" t="n">
+        <v>2019</v>
+      </c>
+      <c r="J322" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-01-V6</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Tiguan X 2021-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D323" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>BSD-VW-01</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>Tiguan X</t>
+        </is>
+      </c>
+      <c r="I323" t="n">
+        <v>2021</v>
+      </c>
+      <c r="J323" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-01-V7</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen THARU 2019-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D324" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>BSD-VW-01</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>THARU</t>
+        </is>
+      </c>
+      <c r="I324" t="n">
+        <v>2019</v>
+      </c>
+      <c r="J324" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-01-V8</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen T-Cross 2019-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C325" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D325" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>BSD-VW-01</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>T-Cross</t>
+        </is>
+      </c>
+      <c r="I325" t="n">
+        <v>2019</v>
+      </c>
+      <c r="J325" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-01-V9</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Viloran 2020-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C326" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D326" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>BSD-VW-01</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>Viloran</t>
+        </is>
+      </c>
+      <c r="I326" t="n">
+        <v>2020</v>
+      </c>
+      <c r="J326" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-01-V10</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Viloran Electric 2021-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C327" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D327" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>BSD-VW-01</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>Viloran Electric</t>
+        </is>
+      </c>
+      <c r="I327" t="n">
+        <v>2021</v>
+      </c>
+      <c r="J327" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-02-V11</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen T-ROC 2016-2022 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C328" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D328" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>BSD-VW-02</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>T-ROC</t>
+        </is>
+      </c>
+      <c r="I328" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J328" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-03-V12</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Tiguan 2018-2018 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C329" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D329" t="n">
+        <v>900</v>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>BSD-VW-03</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>Tiguan</t>
+        </is>
+      </c>
+      <c r="I329" t="n">
+        <v>2018</v>
+      </c>
+      <c r="J329" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-03-V13</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Lavida 2013-2018 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C330" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D330" t="n">
+        <v>900</v>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>BSD-VW-03</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>Lavida</t>
+        </is>
+      </c>
+      <c r="I330" t="n">
+        <v>2013</v>
+      </c>
+      <c r="J330" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-03-V14</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Jetta 2011-2011 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C331" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D331" t="n">
+        <v>900</v>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>BSD-VW-03</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>Jetta</t>
+        </is>
+      </c>
+      <c r="I331" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J331" t="n">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-04-V15</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Golf 8 2021-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C332" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D332" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>BSD-VW-04</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>Golf 8</t>
+        </is>
+      </c>
+      <c r="I332" t="n">
+        <v>2021</v>
+      </c>
+      <c r="J332" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-04-V16</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen ID.3 2021-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C333" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D333" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>BSD-VW-04</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>ID.3</t>
+        </is>
+      </c>
+      <c r="I333" t="n">
+        <v>2021</v>
+      </c>
+      <c r="J333" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-04-V17</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Lamando L 2023-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C334" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D334" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>BSD-VW-04</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>Lamando L</t>
+        </is>
+      </c>
+      <c r="I334" t="n">
+        <v>2023</v>
+      </c>
+      <c r="J334" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-05-V18</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Magotan 2017-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C335" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D335" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>BSD-VW-05</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>Magotan</t>
+        </is>
+      </c>
+      <c r="I335" t="n">
+        <v>2017</v>
+      </c>
+      <c r="J335" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-05-V19</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen CC 2018-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C336" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D336" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>BSD-VW-05</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="I336" t="n">
+        <v>2018</v>
+      </c>
+      <c r="J336" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-05-V20</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Magotan GTE 2020-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C337" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D337" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>BSD-VW-05</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>Magotan GTE</t>
+        </is>
+      </c>
+      <c r="I337" t="n">
+        <v>2020</v>
+      </c>
+      <c r="J337" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-05-V21</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Passat Variant 2016-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C338" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D338" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>BSD-VW-05</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>Passat Variant</t>
+        </is>
+      </c>
+      <c r="I338" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J338" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-06-V22</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Golf 7 2014-2020 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C339" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D339" t="n">
+        <v>900</v>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>BSD-VW-06</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>Golf 7</t>
+        </is>
+      </c>
+      <c r="I339" t="n">
+        <v>2014</v>
+      </c>
+      <c r="J339" t="n">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-06-V23</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Golf Electric 2020-2020 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C340" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D340" t="n">
+        <v>900</v>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>BSD-VW-06</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>Golf Electric</t>
+        </is>
+      </c>
+      <c r="I340" t="n">
+        <v>2020</v>
+      </c>
+      <c r="J340" t="n">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-06-V24</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Touran L 2016-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C341" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D341" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>BSD-VW-06</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>Touran L</t>
+        </is>
+      </c>
+      <c r="I341" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J341" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-06-V25</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Lamando 2015-2018 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C342" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D342" t="n">
+        <v>900</v>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>BSD-VW-06</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>Lamando</t>
+        </is>
+      </c>
+      <c r="I342" t="n">
+        <v>2015</v>
+      </c>
+      <c r="J342" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-07-V26</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Golf 6 2010-2013 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C343" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D343" t="n">
+        <v>900</v>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>BSD-VW-07</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>Golf 6</t>
+        </is>
+      </c>
+      <c r="I343" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J343" t="n">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-07-V27</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Bora 2011-2016 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C344" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D344" t="n">
+        <v>900</v>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>BSD-VW-07</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>Bora</t>
+        </is>
+      </c>
+      <c r="I344" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J344" t="n">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-07-V28</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Touran 2011-2015 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C345" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D345" t="n">
+        <v>900</v>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>BSD-VW-07</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>Touran</t>
+        </is>
+      </c>
+      <c r="I345" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J345" t="n">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-07-V29</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Passat 2009-2010 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C346" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D346" t="n">
+        <v>900</v>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>BSD-VW-07</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>Passat</t>
+        </is>
+      </c>
+      <c r="I346" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J346" t="n">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-08-V30</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Bora 2019-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C347" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D347" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>BSD-VW-08</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>Bora</t>
+        </is>
+      </c>
+      <c r="I347" t="n">
+        <v>2019</v>
+      </c>
+      <c r="J347" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-08-V31</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Sagitar 2019-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C348" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D348" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>BSD-VW-08</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>Sagitar</t>
+        </is>
+      </c>
+      <c r="I348" t="n">
+        <v>2019</v>
+      </c>
+      <c r="J348" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-08-V32</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Lavida PLUS 2018-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C349" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D349" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>BSD-VW-08</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>Lavida PLUS</t>
+        </is>
+      </c>
+      <c r="I349" t="n">
+        <v>2018</v>
+      </c>
+      <c r="J349" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-08-V33</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Lamando 2012-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C350" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D350" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>BSD-VW-08</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>Lamando</t>
+        </is>
+      </c>
+      <c r="I350" t="n">
+        <v>2012</v>
+      </c>
+      <c r="J350" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-08-V34</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Passat 2019-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C351" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D351" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>BSD-VW-08</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>Passat</t>
+        </is>
+      </c>
+      <c r="I351" t="n">
+        <v>2019</v>
+      </c>
+      <c r="J351" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-09-V35</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Bora 2016-2018 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C352" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D352" t="n">
+        <v>900</v>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>BSD-VW-09</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>Bora</t>
+        </is>
+      </c>
+      <c r="I352" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J352" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-09-V36</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Sagitar 2017-2018 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C353" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D353" t="n">
+        <v>900</v>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>BSD-VW-09</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>Sagitar</t>
+        </is>
+      </c>
+      <c r="I353" t="n">
+        <v>2017</v>
+      </c>
+      <c r="J353" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-09-V37</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen C-TREK 2017-2023 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C354" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D354" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>BSD-VW-09</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>C-TREK</t>
+        </is>
+      </c>
+      <c r="I354" t="n">
+        <v>2017</v>
+      </c>
+      <c r="J354" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-10-V38</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Magotan 2012-2016 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C355" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D355" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>BSD-VW-10</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>Magotan</t>
+        </is>
+      </c>
+      <c r="I355" t="n">
+        <v>2012</v>
+      </c>
+      <c r="J355" t="n">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-10-V39</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen CC 2010-2018 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C356" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D356" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>BSD-VW-10</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="I356" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J356" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-10-V40</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Beetle 2002-2002 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C357" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D357" t="n">
+        <v>900</v>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>BSD-VW-10</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>Beetle</t>
+        </is>
+      </c>
+      <c r="I357" t="n">
+        <v>2002</v>
+      </c>
+      <c r="J357" t="n">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-10-V41</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Scirocco 2009-2016 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C358" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D358" t="n">
+        <v>900</v>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>BSD-VW-10</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>Scirocco</t>
+        </is>
+      </c>
+      <c r="I358" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J358" t="n">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-11-V42</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Passat 2011-2018 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C359" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D359" t="n">
+        <v>900</v>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>BSD-VW-11</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>Passat</t>
+        </is>
+      </c>
+      <c r="I359" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J359" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-12-V43</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Golf Sportsvan 2016-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C360" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D360" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>BSD-VW-12</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>Golf Sportsvan</t>
+        </is>
+      </c>
+      <c r="I360" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J360" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-12-V44</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen ID.4 CROZZ 2021-2023 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C361" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D361" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>BSD-VW-12</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>ID.4 CROZZ</t>
+        </is>
+      </c>
+      <c r="I361" t="n">
+        <v>2021</v>
+      </c>
+      <c r="J361" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-12-V45</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen ID.6 CROZZ 2021-2023 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C362" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D362" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>BSD-VW-12</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>ID.6 CROZZ</t>
+        </is>
+      </c>
+      <c r="I362" t="n">
+        <v>2021</v>
+      </c>
+      <c r="J362" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-12-V46</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen ID.4X 2021-2023 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C363" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D363" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>BSD-VW-12</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>ID.4X</t>
+        </is>
+      </c>
+      <c r="I363" t="n">
+        <v>2021</v>
+      </c>
+      <c r="J363" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-12-V47</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen ID.6X 2021-2023 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C364" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D364" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>BSD-VW-12</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>ID.6X</t>
+        </is>
+      </c>
+      <c r="I364" t="n">
+        <v>2021</v>
+      </c>
+      <c r="J364" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-12-V48</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen ID.5 2022-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C365" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D365" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>BSD-VW-12</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>ID.5</t>
+        </is>
+      </c>
+      <c r="I365" t="n">
+        <v>2022</v>
+      </c>
+      <c r="J365" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-13-V49</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen T-ROC 2018-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C366" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D366" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>BSD-VW-13</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>T-ROC</t>
+        </is>
+      </c>
+      <c r="I366" t="n">
+        <v>2018</v>
+      </c>
+      <c r="J366" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-13-V50</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Lavida 2023-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C367" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D367" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>BSD-VW-13</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>Lavida</t>
+        </is>
+      </c>
+      <c r="I367" t="n">
+        <v>2023</v>
+      </c>
+      <c r="J367" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-13-V51</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Lavida 2008-2012 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C368" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D368" t="n">
+        <v>900</v>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>BSD-VW-13</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>Lavida</t>
+        </is>
+      </c>
+      <c r="I368" t="n">
+        <v>2008</v>
+      </c>
+      <c r="J368" t="n">
+        <v>2012</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-13-V52</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Lavida Typical 2013-2013 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C369" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D369" t="n">
+        <v>900</v>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>BSD-VW-13</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>Lavida Typical</t>
+        </is>
+      </c>
+      <c r="I369" t="n">
+        <v>2013</v>
+      </c>
+      <c r="J369" t="n">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-13-V53</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Magotan 2001-2010 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C370" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D370" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>BSD-VW-13</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>Magotan</t>
+        </is>
+      </c>
+      <c r="I370" t="n">
+        <v>2001</v>
+      </c>
+      <c r="J370" t="n">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-14-V54</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Gran Lavida 2013-2014 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C371" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D371" t="n">
+        <v>900</v>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>BSD-VW-14</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>Gran Lavida</t>
+        </is>
+      </c>
+      <c r="I371" t="n">
+        <v>2013</v>
+      </c>
+      <c r="J371" t="n">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-14-V55</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen POLO 2014-2018 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C372" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D372" t="n">
+        <v>900</v>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>BSD-VW-14</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>POLO</t>
+        </is>
+      </c>
+      <c r="I372" t="n">
+        <v>2014</v>
+      </c>
+      <c r="J372" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-14-V56</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Lavida 2016-2017 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C373" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D373" t="n">
+        <v>900</v>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>BSD-VW-14</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>Lavida</t>
+        </is>
+      </c>
+      <c r="I373" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J373" t="n">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-14-V57</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Jetta 2017-2019 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C374" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D374" t="n">
+        <v>900</v>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>BSD-VW-14</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>Jetta</t>
+        </is>
+      </c>
+      <c r="I374" t="n">
+        <v>2017</v>
+      </c>
+      <c r="J374" t="n">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-15-V58</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Santana 2016-2022 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C375" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D375" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>BSD-VW-15</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>Santana</t>
+        </is>
+      </c>
+      <c r="I375" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J375" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-15-V59</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Cross Lavida 2015-2022 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C376" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D376" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>BSD-VW-15</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>Cross Lavida</t>
+        </is>
+      </c>
+      <c r="I376" t="n">
+        <v>2015</v>
+      </c>
+      <c r="J376" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-15-V60</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Cross Santana 2017-2022 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C377" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D377" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>BSD-VW-15</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>Cross Santana</t>
+        </is>
+      </c>
+      <c r="I377" t="n">
+        <v>2017</v>
+      </c>
+      <c r="J377" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-16-V61</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Tiguan 2010-2017 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C378" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D378" t="n">
+        <v>900</v>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>BSD-VW-16</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>Tiguan</t>
+        </is>
+      </c>
+      <c r="I378" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J378" t="n">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-16-V62</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Sharan 2012-2022 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C379" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D379" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>BSD-VW-16</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>Sharan</t>
+        </is>
+      </c>
+      <c r="I379" t="n">
+        <v>2012</v>
+      </c>
+      <c r="J379" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-17-V63</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Teramont 2017-2023 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C380" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D380" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>BSD-VW-17</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>Teramont</t>
+        </is>
+      </c>
+      <c r="I380" t="n">
+        <v>2017</v>
+      </c>
+      <c r="J380" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-17-V64</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Teramont X 2017-2023 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C381" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D381" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>BSD-VW-17</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>Teramont X</t>
+        </is>
+      </c>
+      <c r="I381" t="n">
+        <v>2017</v>
+      </c>
+      <c r="J381" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-17-V65</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Santana 2013-2023 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C382" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D382" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>BSD-VW-17</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>Santana</t>
+        </is>
+      </c>
+      <c r="I382" t="n">
+        <v>2013</v>
+      </c>
+      <c r="J382" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-18-V66</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Jetta 2018-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C383" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D383" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>BSD-VW-18</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>Jetta</t>
+        </is>
+      </c>
+      <c r="I383" t="n">
+        <v>2018</v>
+      </c>
+      <c r="J383" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-19-V67</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen POLO PLUS 2019-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C384" t="n">
+        <v>1399</v>
+      </c>
+      <c r="D384" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>BSD-VW-19</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>POLO PLUS</t>
+        </is>
+      </c>
+      <c r="I384" t="n">
+        <v>2019</v>
+      </c>
+      <c r="J384" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-20-V68</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen PHIDEON 2016-2024 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C385" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D385" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>BSD-VW-20</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>PHIDEON</t>
+        </is>
+      </c>
+      <c r="I385" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J385" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-21-V69</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Touareg 2014-2018 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C386" t="n">
+        <v>1599</v>
+      </c>
+      <c r="D386" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>BSD-VW-21</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>Touareg</t>
+        </is>
+      </c>
+      <c r="I386" t="n">
+        <v>2014</v>
+      </c>
+      <c r="J386" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>BSD-01+BSD-VW-22-V70</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Senzor unghi mort Volkswagen Touareg 2019-2023 — oglindă dedicată</t>
+        </is>
+      </c>
+      <c r="C387" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D387" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>BSD-01</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>BSD-VW-22</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>Touareg</t>
+        </is>
+      </c>
+      <c r="I387" t="n">
+        <v>2019</v>
+      </c>
+      <c r="J387" t="n">
+        <v>2023</v>
       </c>
     </row>
   </sheetData>

</xml_diff>